<commit_message>
Auto pipeline update 2026-04-28 16:08:54
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -3872,7 +3872,7 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-04-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3959,7 +3959,7 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-04-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -4046,7 +4046,7 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-04-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -4129,7 +4129,7 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-04-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -4212,7 +4212,7 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-04-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -4295,7 +4295,7 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-04-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4390,7 +4390,7 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-04-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -4477,7 +4477,7 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-04-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -4543,7 +4543,7 @@
       </c>
       <c r="Y46" t="inlineStr">
         <is>
-          <t>25/0, 33/0, 54/5,62/0, 63B/0, 63B/1 64/1, 64A/0, 78/2</t>
+          <t>25/0, 33/0, 54/5,62/0, 63B/0, 63B/1 64/1,78/2</t>
         </is>
       </c>
     </row>
@@ -4572,7 +4572,7 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-04-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -4661,7 +4661,7 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-04-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -4740,7 +4740,7 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-04-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -4823,7 +4823,7 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-04-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -4906,7 +4906,7 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-04-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -4989,7 +4989,7 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-04-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -9898,7 +9898,7 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -9995,7 +9995,7 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
@@ -10092,7 +10092,7 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -10189,7 +10189,7 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -10282,7 +10282,7 @@
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
@@ -10332,16 +10332,14 @@
         <v>33</v>
       </c>
       <c r="T112" t="n">
-        <v>11</v>
-      </c>
-      <c r="U112" t="n">
-        <v>1</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="U112" t="inlineStr"/>
       <c r="V112" t="n">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="W112" t="n">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="X112" t="inlineStr">
         <is>
@@ -10383,7 +10381,7 @@
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -10480,7 +10478,7 @@
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -10532,9 +10530,7 @@
       <c r="T114" t="n">
         <v>5</v>
       </c>
-      <c r="U114" t="n">
-        <v>1</v>
-      </c>
+      <c r="U114" t="inlineStr"/>
       <c r="V114" t="n">
         <v>193</v>
       </c>
@@ -10548,7 +10544,7 @@
       </c>
       <c r="Y114" t="inlineStr">
         <is>
-          <t>Today com - 10/7             WIP - 8/1 &amp; 7/7</t>
+          <t>WIP - 8/1 , 7/7, 92/0</t>
         </is>
       </c>
     </row>
@@ -10581,7 +10577,7 @@
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -10634,7 +10630,7 @@
         <v>19</v>
       </c>
       <c r="U115" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V115" t="n">
         <v>80</v>
@@ -10649,7 +10645,7 @@
       </c>
       <c r="Y115" t="inlineStr">
         <is>
-          <t>Today Com -134A/1      WIP - 134A/0</t>
+          <t>Today Com -134A/3       WIP - 136/0</t>
         </is>
       </c>
     </row>
@@ -10682,7 +10678,7 @@
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -10757,7 +10753,7 @@
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -10823,7 +10819,7 @@
       </c>
       <c r="Y117" t="inlineStr">
         <is>
-          <t>Today Com-NIL                    WIP- 150/0-151/0 Rly Crossing and 151/0-152/0 Under Preparetion</t>
+          <t>Today Com-NIL                    WIP- 150/0-151/0 Rly Crossing and 151/0-152/0  Preparetion Done.</t>
         </is>
       </c>
     </row>
@@ -10856,7 +10852,7 @@
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -10951,7 +10947,7 @@
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -11034,7 +11030,7 @@
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -11119,7 +11115,7 @@
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -11204,7 +11200,7 @@
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -11297,7 +11293,7 @@
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -11390,7 +11386,7 @@
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -11483,7 +11479,7 @@
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -11576,7 +11572,7 @@
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -11677,7 +11673,7 @@
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -11770,7 +11766,7 @@
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -11820,25 +11816,21 @@
         <v>7</v>
       </c>
       <c r="T128" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U128" t="n">
         <v>0</v>
       </c>
       <c r="V128" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W128" t="n">
-        <v>41</v>
-      </c>
-      <c r="X128" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="X128" t="inlineStr"/>
       <c r="Y128" t="inlineStr">
         <is>
-          <t>Today Complete-Nil              WIP -2/1 (LO)</t>
+          <t>After Completion 2/1, Gang shifted at 400kV</t>
         </is>
       </c>
     </row>
@@ -11871,7 +11863,7 @@
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -11956,7 +11948,7 @@
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -12033,7 +12025,7 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -12120,7 +12112,7 @@
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -12207,7 +12199,7 @@
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -12599,7 +12591,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-04-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -12634,7 +12626,7 @@
       <c r="I6" t="inlineStr">
         <is>
           <t>C3:Activity-&gt;activity_raw; C4:Quantity-&gt;quantity_loa; C5:unnamed_col_5-&gt;quantity_estimated_or_total; C7:unnamed_col_7-&gt;cumulative_last_month; C9:unnamed_col_9-&gt;plan_for_month; C10:Progress for the Month-&gt;progress_for_month; C11:unnamed_col_11-&gt;today_progress; C12:Cumulative Progress-&gt;cumulative_progress; C13:Balance Progress-&gt;balance_progress; C14:Gangs working 
-Apr-26-&gt;gangs_working; C15:2026-04-26 00:00:00 Remarks-&gt;remarks</t>
+Apr-26-&gt;gangs_working; C15:2026-04-27 00:00:00 Remarks-&gt;remarks</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -13011,7 +13003,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -13073,7 +13065,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -13143,9 +13135,52 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Workbook</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ConfiguredSheet</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>LineName</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>LineNameSource</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13495,7 +13530,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-04-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -14007,7 +14042,7 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -14053,7 +14088,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-04-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-04-27.xlsx</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">

</xml_diff>

<commit_message>
Auto pipeline update 2026-04-29 11:43:51
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -3508,7 +3508,7 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-04-25.xlsx</t>
+          <t>TA 418 - DPR - 2026-04-29.xlsx</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -3599,7 +3599,7 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-04-25.xlsx</t>
+          <t>TA 418 - DPR - 2026-04-29.xlsx</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3690,7 +3690,7 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-04-25.xlsx</t>
+          <t>TA 418 - DPR - 2026-04-29.xlsx</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3781,7 +3781,7 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-04-25.xlsx</t>
+          <t>TA 418 - DPR - 2026-04-29.xlsx</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -5060,7 +5060,7 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-04-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-04-28.xlsx</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -5147,7 +5147,7 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-04-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-04-28.xlsx</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -5232,7 +5232,7 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-04-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-04-28.xlsx</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -5319,7 +5319,7 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-04-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-04-28.xlsx</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -5365,16 +5365,16 @@
       </c>
       <c r="S56" t="inlineStr"/>
       <c r="T56" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="U56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V56" t="n">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="W56" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="X56" t="inlineStr">
         <is>
@@ -5383,7 +5383,7 @@
       </c>
       <c r="Y56" t="inlineStr">
         <is>
-          <t>WIP - 36/4 , 5</t>
+          <t>WIP - 36/4 , 5  &amp; 4/14</t>
         </is>
       </c>
     </row>
@@ -5412,7 +5412,7 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-04-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-04-28.xlsx</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -5503,7 +5503,7 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-04-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-04-28.xlsx</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="Y58" t="inlineStr">
         <is>
-          <t>42/0 - 43/0 -  pilot payingout  done(work has been interrupted today due to Rain) + 35/0 - 36/0 - Insulator hosting under Progress</t>
+          <t>42/0 - 43/0 -  Pilot payingout  Completed  + 35/0 - 36/0 - Insulator hosting under Progress</t>
         </is>
       </c>
     </row>
@@ -5596,7 +5596,7 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-04-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-04-28.xlsx</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -5654,7 +5654,11 @@
         <v>17.80000000000001</v>
       </c>
       <c r="X59" t="inlineStr"/>
-      <c r="Y59" t="inlineStr"/>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>Top Final sag planned for tomorrow</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5681,7 +5685,7 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-04-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-04-28.xlsx</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -5766,7 +5770,7 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-04-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-04-28.xlsx</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -5845,7 +5849,7 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-04-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-04-28.xlsx</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -12534,7 +12538,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-04-25.xlsx</t>
+          <t>TA 418 - DPR - 2026-04-29.xlsx</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -12653,7 +12657,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-04-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-04-28.xlsx</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -13484,7 +13488,7 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-04-25.xlsx</t>
+          <t>TA 418 - DPR - 2026-04-29.xlsx</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -13576,7 +13580,7 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-04-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-04-28.xlsx</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -13802,7 +13806,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-04-27.xlsx</t>
+          <t>TA 512 - DPR - 2026-04-28.xlsx</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -14138,7 +14142,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-04-27.xlsx</t>
+          <t>TB 605 - DPR - 2026-04-28.xlsx</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>

</xml_diff>

<commit_message>
Publish snapshot part 2 (parquets)
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -592,12 +592,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -682,12 +682,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -772,12 +772,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -862,12 +862,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -952,12 +952,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1005,16 +1005,16 @@
         <v>34</v>
       </c>
       <c r="U6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="V6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W6" t="n">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="X6" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
@@ -1052,12 +1052,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1105,16 +1105,16 @@
         <v>34</v>
       </c>
       <c r="U7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="V7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W7" t="n">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="X7" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
@@ -1152,12 +1152,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1205,14 +1205,14 @@
         <v>34</v>
       </c>
       <c r="U8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="n">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="X8" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr"/>
@@ -1246,12 +1246,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1299,25 +1299,23 @@
         <v>55</v>
       </c>
       <c r="U9" t="n">
-        <v>5</v>
-      </c>
-      <c r="V9" t="n">
-        <v>1</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="V9" t="inlineStr"/>
       <c r="W9" t="n">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="X9" t="n">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>13.0</t>
+          <t>14.0</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>1 gang arrived on 02.05.26</t>
+          <t>1 gang arrived on 07.05.26</t>
         </is>
       </c>
     </row>
@@ -1350,12 +1348,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1403,16 +1401,16 @@
         <v>55</v>
       </c>
       <c r="U10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V10" t="n">
         <v>0</v>
       </c>
       <c r="W10" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="X10" t="n">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
@@ -1450,12 +1448,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1507,14 +1505,14 @@
       </c>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="n">
-        <v>6.628</v>
+        <v>7.096</v>
       </c>
       <c r="X11" t="n">
-        <v>121.171</v>
+        <v>120.703</v>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr"/>
@@ -1548,12 +1546,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1640,12 +1638,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1692,13 +1690,15 @@
       <c r="T13" t="n">
         <v>20</v>
       </c>
-      <c r="U13" t="inlineStr"/>
+      <c r="U13" t="n">
+        <v>0.468001</v>
+      </c>
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="n">
-        <v>6.628</v>
+        <v>7.096</v>
       </c>
       <c r="X13" t="n">
-        <v>121.171</v>
+        <v>120.703</v>
       </c>
       <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="inlineStr"/>
@@ -1732,12 +1732,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1824,12 +1824,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1924,12 +1924,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2024,12 +2024,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2124,12 +2124,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2224,12 +2224,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-05-04.xlsx</t>
+          <t>TA 418 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2324,12 +2324,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-05-04.xlsx</t>
+          <t>TA 418 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2377,16 +2377,16 @@
         <v>1</v>
       </c>
       <c r="U20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V20" t="n">
         <v>0</v>
       </c>
       <c r="W20" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="X20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
@@ -2424,12 +2424,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-05-04.xlsx</t>
+          <t>TA 418 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2524,12 +2524,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-05-04.xlsx</t>
+          <t>TA 418 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2579,9 +2579,7 @@
       <c r="U22" t="n">
         <v>2.704</v>
       </c>
-      <c r="V22" t="n">
-        <v>2.704</v>
-      </c>
+      <c r="V22" t="inlineStr"/>
       <c r="W22" t="n">
         <v>26.446</v>
       </c>
@@ -2624,12 +2622,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2720,12 +2718,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2816,12 +2814,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2908,12 +2906,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -3000,12 +2998,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -3092,12 +3090,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -3147,14 +3145,14 @@
         <v>45</v>
       </c>
       <c r="U28" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="V28" t="inlineStr"/>
       <c r="W28" t="n">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="X28" t="n">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
@@ -3163,7 +3161,7 @@
       </c>
       <c r="Z28" t="inlineStr">
         <is>
-          <t>37/0, 38/2, 38/3, 41/2, 52/1, 53/0, 54/0, 52/0, 59/0, 61/0, 64/4, 65/0, 68/0, 67/0, 69/0, 70/0,  71/0, 84/2, 87/1, 87/2</t>
+          <t>37/0, 38/2, 38/3, 52/1, 52/2, 54/0, 52/0, 59/0, 65/0, 66/0, 67/0, 69/0, 70/0,  71/0, 87/1, 87/2, 72/0, 73/0</t>
         </is>
       </c>
     </row>
@@ -3196,12 +3194,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3292,12 +3290,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -3347,14 +3345,14 @@
         <v>40</v>
       </c>
       <c r="U30" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="V30" t="inlineStr"/>
       <c r="W30" t="n">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="X30" t="n">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
@@ -3363,7 +3361,7 @@
       </c>
       <c r="Z30" t="inlineStr">
         <is>
-          <t>14/0,33/0,62/0, 63B/0, 63B/1 64/1,64/5, 81/0</t>
+          <t>13/0, 14/0, 14/1, 40/8, 42/0 , 62/0,  64/2, 64/3, 81/0</t>
         </is>
       </c>
     </row>
@@ -3396,12 +3394,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3494,12 +3492,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3582,12 +3580,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3674,12 +3672,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3766,12 +3764,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3858,12 +3856,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3938,12 +3936,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-03.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -4034,12 +4032,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-03.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -4128,12 +4126,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-03.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -4224,12 +4222,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-03.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -4276,17 +4274,19 @@
       <c r="T40" t="n">
         <v>40</v>
       </c>
-      <c r="U40" t="inlineStr"/>
+      <c r="U40" t="n">
+        <v>7</v>
+      </c>
       <c r="V40" t="inlineStr"/>
       <c r="W40" t="n">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="X40" t="n">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="Z40" t="inlineStr"/>
@@ -4320,12 +4320,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-03.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -4372,17 +4372,21 @@
       <c r="T41" t="n">
         <v>24</v>
       </c>
-      <c r="U41" t="inlineStr"/>
-      <c r="V41" t="inlineStr"/>
+      <c r="U41" t="n">
+        <v>5</v>
+      </c>
+      <c r="V41" t="n">
+        <v>1</v>
+      </c>
       <c r="W41" t="n">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="X41" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="Y41" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="Z41" t="inlineStr"/>
@@ -4416,12 +4420,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-03.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4468,13 +4472,15 @@
       <c r="T42" t="n">
         <v>14.192</v>
       </c>
-      <c r="U42" t="inlineStr"/>
+      <c r="U42" t="n">
+        <v>3.949</v>
+      </c>
       <c r="V42" t="inlineStr"/>
       <c r="W42" t="n">
-        <v>107.15</v>
+        <v>111.099</v>
       </c>
       <c r="X42" t="n">
-        <v>14.19199999999999</v>
+        <v>10.24299999999999</v>
       </c>
       <c r="Y42" t="inlineStr">
         <is>
@@ -4483,7 +4489,7 @@
       </c>
       <c r="Z42" t="inlineStr">
         <is>
-          <t>42/0 - 43/0 -  Middle  phase  Rough sag done    + 35/0 - 36/0 - Insulator hosting under Progress</t>
+          <t>35/0 - 36/0 - Insulator hosting  Done  + 43/0 - 43A/0 - Insulator Hosting under progress</t>
         </is>
       </c>
     </row>
@@ -4516,12 +4522,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-03.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4568,13 +4574,17 @@
       <c r="T43" t="n">
         <v>14.192</v>
       </c>
-      <c r="U43" t="inlineStr"/>
-      <c r="V43" t="inlineStr"/>
+      <c r="U43" t="n">
+        <v>3.949</v>
+      </c>
+      <c r="V43" t="n">
+        <v>3.949</v>
+      </c>
       <c r="W43" t="n">
-        <v>107.15</v>
+        <v>111.099</v>
       </c>
       <c r="X43" t="n">
-        <v>14.19199999999999</v>
+        <v>10.24299999999999</v>
       </c>
       <c r="Y43" t="inlineStr"/>
       <c r="Z43" t="inlineStr"/>
@@ -4608,12 +4618,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-03.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4700,12 +4710,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-03.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4788,12 +4798,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-03.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4876,12 +4886,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-10.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -4966,12 +4976,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-10.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -5058,12 +5068,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-10.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -5152,12 +5162,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-10.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -5244,12 +5254,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-10.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -5336,12 +5346,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-10.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -5424,12 +5434,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>TA 505 - DPR - 2026-04-17.xlsx</t>
+          <t>TA 505 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -5512,12 +5522,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>TA 505 - DPR - 2026-04-17.xlsx</t>
+          <t>TA 505 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5600,12 +5610,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>TA 505 - DPR - 2026-04-17.xlsx</t>
+          <t>TA 505 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -5647,25 +5657,25 @@
         <v>379</v>
       </c>
       <c r="S55" t="n">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="T55" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="U55" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V55" t="inlineStr"/>
       <c r="W55" t="n">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="X55" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="Y55" t="inlineStr"/>
       <c r="Z55" t="inlineStr">
         <is>
-          <t>6 Locations are under severe RoW.</t>
+          <t>5 Locations are under severe RoW.</t>
         </is>
       </c>
     </row>
@@ -5698,12 +5708,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>TA 505 - DPR - 2026-04-17.xlsx</t>
+          <t>TA 505 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -5745,23 +5755,27 @@
         <v>379</v>
       </c>
       <c r="S56" t="n">
-        <v>321</v>
+        <v>347</v>
       </c>
       <c r="T56" t="n">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="U56" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="V56" t="inlineStr"/>
       <c r="W56" t="n">
-        <v>338</v>
+        <v>351</v>
       </c>
       <c r="X56" t="n">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="Y56" t="inlineStr"/>
-      <c r="Z56" t="inlineStr"/>
+      <c r="Z56" t="inlineStr">
+        <is>
+          <t>Tack Welding Completed- 98/339,                Gangs Engaged-3.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5792,12 +5806,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>TA 505 - DPR - 2026-04-17.xlsx</t>
+          <t>TA 505 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -5839,20 +5853,20 @@
         <v>139.6</v>
       </c>
       <c r="S57" t="n">
-        <v>13.039</v>
+        <v>14.006</v>
       </c>
       <c r="T57" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="U57" t="n">
-        <v>0.9670000000000005</v>
+        <v>0</v>
       </c>
       <c r="V57" t="inlineStr"/>
       <c r="W57" t="n">
         <v>14.006</v>
       </c>
       <c r="X57" t="n">
-        <v>126.561</v>
+        <v>125.594</v>
       </c>
       <c r="Y57" t="inlineStr"/>
       <c r="Z57" t="inlineStr"/>
@@ -5886,12 +5900,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>TA 505 - DPR - 2026-04-17.xlsx</t>
+          <t>TA 505 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -5936,7 +5950,7 @@
         <v>14.006</v>
       </c>
       <c r="T58" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="U58" t="n">
         <v>0</v>
@@ -5980,12 +5994,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-10.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -6070,12 +6084,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-10.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -6160,12 +6174,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-10.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -6254,12 +6268,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-10.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -6346,12 +6360,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-10.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -6440,12 +6454,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-10.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -6524,12 +6538,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>TA 509 - DPR - 2026-01-17.xlsx</t>
+          <t>TA 509 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -6573,24 +6587,24 @@
         <v>309</v>
       </c>
       <c r="S65" t="n">
-        <v>228</v>
+        <v>258</v>
       </c>
       <c r="T65" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="U65" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V65" t="inlineStr"/>
       <c r="W65" t="n">
-        <v>231</v>
+        <v>262</v>
       </c>
       <c r="X65" t="n">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="Y65" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="Z65" t="inlineStr"/>
@@ -6624,12 +6638,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>TA 509 - DPR - 2026-01-17.xlsx</t>
+          <t>TA 509 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -6673,26 +6687,22 @@
         <v>309</v>
       </c>
       <c r="S66" t="n">
-        <v>189</v>
+        <v>228</v>
       </c>
       <c r="T66" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="U66" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V66" t="inlineStr"/>
       <c r="W66" t="n">
-        <v>191</v>
+        <v>231</v>
       </c>
       <c r="X66" t="n">
-        <v>118</v>
-      </c>
-      <c r="Y66" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="Y66" t="inlineStr"/>
       <c r="Z66" t="inlineStr"/>
     </row>
     <row r="67">
@@ -6724,12 +6734,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>TA 509 - DPR - 2026-01-17.xlsx</t>
+          <t>TA 509 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -6773,24 +6783,24 @@
         <v>309</v>
       </c>
       <c r="S67" t="n">
-        <v>59</v>
+        <v>180</v>
       </c>
       <c r="T67" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="U67" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="V67" t="inlineStr"/>
       <c r="W67" t="n">
-        <v>69</v>
+        <v>186</v>
       </c>
       <c r="X67" t="n">
-        <v>240</v>
+        <v>123</v>
       </c>
       <c r="Y67" t="inlineStr">
         <is>
-          <t>7.0</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="Z67" t="inlineStr"/>
@@ -6824,12 +6834,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>TA 509 - DPR - 2026-01-17.xlsx</t>
+          <t>TA 509 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -6918,12 +6928,12 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -7014,12 +7024,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -7110,12 +7120,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -7206,12 +7216,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -7302,12 +7312,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -7398,12 +7408,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -7450,17 +7460,21 @@
       <c r="T74" t="n">
         <v>272</v>
       </c>
-      <c r="U74" t="inlineStr"/>
+      <c r="U74" t="n">
+        <v>1</v>
+      </c>
       <c r="V74" t="n">
         <v>25</v>
       </c>
-      <c r="W74" t="inlineStr"/>
+      <c r="W74" t="n">
+        <v>0</v>
+      </c>
       <c r="X74" t="n">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="Y74" t="inlineStr">
         <is>
-          <t>03/24</t>
+          <t>02/17</t>
         </is>
       </c>
       <c r="Z74" t="inlineStr"/>
@@ -7494,12 +7508,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -7582,12 +7596,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -7641,7 +7655,7 @@
         <v>30</v>
       </c>
       <c r="W76" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X76" t="n">
         <v>215</v>
@@ -7682,12 +7696,12 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -7735,14 +7749,14 @@
         <v>0</v>
       </c>
       <c r="U77" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="V77" t="inlineStr"/>
       <c r="W77" t="n">
         <v>2</v>
       </c>
       <c r="X77" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="Y77" t="inlineStr"/>
       <c r="Z77" t="inlineStr"/>
@@ -7776,12 +7790,12 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -7870,12 +7884,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -7964,12 +7978,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -8058,12 +8072,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -8152,12 +8166,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -8248,12 +8262,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -8344,12 +8358,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -8438,12 +8452,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -8532,12 +8546,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -8626,12 +8640,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -8724,12 +8738,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -8779,16 +8793,16 @@
         <v>350</v>
       </c>
       <c r="U88" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V88" t="n">
         <v>1</v>
       </c>
       <c r="W88" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="X88" t="n">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="Y88" t="inlineStr">
         <is>
@@ -8797,10 +8811,9 @@
       </c>
       <c r="Z88" t="inlineStr">
         <is>
-          <t>Loc-52/1-Pit A , B ,D PCC Compl
-Loc-55/4-Backfilling WIP
-Loc-52/0-Casting compl.
-Loc-52/5-Pit D Steel Binding Compl.</t>
+          <t>Loc-52/1-Casting compl
+Loc-55/3-Pit B Chimney casted ,Pit C Excavation done
+Loc-52/5-Casting WIP</t>
         </is>
       </c>
     </row>
@@ -8833,12 +8846,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -8927,12 +8940,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -8989,8 +9002,16 @@
       <c r="X90" t="n">
         <v>378</v>
       </c>
-      <c r="Y90" t="inlineStr"/>
-      <c r="Z90" t="inlineStr"/>
+      <c r="Y90" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Z90" t="inlineStr">
+        <is>
+          <t>Material Shifting Underprogress</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -9021,12 +9042,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -9115,12 +9136,12 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -9207,12 +9228,12 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -9299,12 +9320,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -9391,12 +9412,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -9485,12 +9506,12 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -9579,12 +9600,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -9673,12 +9694,12 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -9767,12 +9788,12 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -9861,12 +9882,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -9955,12 +9976,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -10053,12 +10074,12 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -10122,7 +10143,7 @@
       </c>
       <c r="Z102" t="inlineStr">
         <is>
-          <t>Loc-30/0-Excavation WIP</t>
+          <t>Loc-30/0-Pit A &amp; D frustum casted</t>
         </is>
       </c>
     </row>
@@ -10155,12 +10176,12 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -10251,12 +10272,12 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -10314,11 +10335,7 @@
         <v>213</v>
       </c>
       <c r="Y104" t="inlineStr"/>
-      <c r="Z104" t="inlineStr">
-        <is>
-          <t>No front Available</t>
-        </is>
-      </c>
+      <c r="Z104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -10349,12 +10366,12 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -10441,12 +10458,12 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -10531,12 +10548,12 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -10619,12 +10636,12 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -10707,12 +10724,12 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -10797,12 +10814,12 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -10853,7 +10870,7 @@
         <v>2</v>
       </c>
       <c r="V110" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W110" t="n">
         <v>115</v>
@@ -10897,12 +10914,12 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -10950,16 +10967,16 @@
         <v>40</v>
       </c>
       <c r="U111" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V111" t="n">
         <v>0</v>
       </c>
       <c r="W111" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="X111" t="n">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="Y111" t="inlineStr"/>
       <c r="Z111" t="inlineStr"/>
@@ -10993,12 +11010,12 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -11089,12 +11106,12 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -11185,12 +11202,12 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -11281,12 +11298,12 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -11377,12 +11394,12 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -11463,12 +11480,12 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -11549,12 +11566,12 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -11635,12 +11652,12 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -11721,12 +11738,12 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -13754,12 +13771,12 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -13856,12 +13873,12 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -13958,12 +13975,12 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -14060,12 +14077,12 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -14162,12 +14179,12 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -14213,27 +14230,27 @@
       <c r="S145" t="n">
         <v>289</v>
       </c>
-      <c r="T145" t="inlineStr"/>
+      <c r="T145" t="n">
+        <v>30</v>
+      </c>
       <c r="U145" t="n">
-        <v>5</v>
-      </c>
-      <c r="V145" t="n">
-        <v>4</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="V145" t="inlineStr"/>
       <c r="W145" t="n">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="X145" t="n">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="Y145" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="Z145" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>60.0</t>
         </is>
       </c>
     </row>
@@ -14270,12 +14287,12 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -14321,18 +14338,20 @@
       <c r="S146" t="n">
         <v>266</v>
       </c>
-      <c r="T146" t="inlineStr"/>
+      <c r="T146" t="n">
+        <v>50</v>
+      </c>
       <c r="U146" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="V146" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W146" t="n">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="X146" t="n">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="Y146" t="inlineStr"/>
       <c r="Z146" t="inlineStr"/>
@@ -14370,12 +14389,12 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -14421,27 +14440,29 @@
       <c r="S147" t="n">
         <v>194</v>
       </c>
-      <c r="T147" t="inlineStr"/>
+      <c r="T147" t="n">
+        <v>30</v>
+      </c>
       <c r="U147" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="V147" t="n">
         <v>1</v>
       </c>
       <c r="W147" t="n">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="X147" t="n">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="Y147" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="Z147" t="inlineStr">
         <is>
-          <t>106.0</t>
+          <t>144.0</t>
         </is>
       </c>
     </row>
@@ -14478,12 +14499,12 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -14533,9 +14554,7 @@
       <c r="U148" t="n">
         <v>7</v>
       </c>
-      <c r="V148" t="n">
-        <v>3</v>
-      </c>
+      <c r="V148" t="inlineStr"/>
       <c r="W148" t="n">
         <v>94</v>
       </c>
@@ -14586,12 +14605,12 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -14670,12 +14689,12 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -14721,7 +14740,9 @@
       <c r="S150" t="n">
         <v>17.483</v>
       </c>
-      <c r="T150" t="inlineStr"/>
+      <c r="T150" t="n">
+        <v>15.147</v>
+      </c>
       <c r="U150" t="n">
         <v>0</v>
       </c>
@@ -14778,12 +14799,12 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -14829,7 +14850,9 @@
       <c r="S151" t="n">
         <v>17.046</v>
       </c>
-      <c r="T151" t="inlineStr"/>
+      <c r="T151" t="n">
+        <v>15.147</v>
+      </c>
       <c r="U151" t="n">
         <v>0</v>
       </c>
@@ -14878,12 +14901,12 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -14970,12 +14993,12 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -15064,12 +15087,12 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -15158,12 +15181,12 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -15260,12 +15283,12 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -15362,12 +15385,12 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -15464,12 +15487,12 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -15566,12 +15589,12 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -15621,16 +15644,14 @@
         <v>0</v>
       </c>
       <c r="U159" t="n">
-        <v>0</v>
-      </c>
-      <c r="V159" t="n">
-        <v>0</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="V159" t="inlineStr"/>
       <c r="W159" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="X159" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="Y159" t="inlineStr">
         <is>
@@ -15676,12 +15697,12 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -15778,12 +15799,12 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -15884,12 +15905,12 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -15978,12 +15999,12 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -16064,12 +16085,12 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -16160,12 +16181,12 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -16256,12 +16277,12 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -16348,12 +16369,12 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-05.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -16446,12 +16467,12 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-05.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -16499,20 +16520,20 @@
         <v>72</v>
       </c>
       <c r="U168" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="V168" t="n">
         <v>0</v>
       </c>
       <c r="W168" t="n">
-        <v>307</v>
+        <v>317</v>
       </c>
       <c r="X168" t="n">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="Y168" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>30</t>
         </is>
       </c>
       <c r="Z168" t="inlineStr"/>
@@ -16546,12 +16567,12 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-05.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -16599,16 +16620,16 @@
         <v>70</v>
       </c>
       <c r="U169" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="V169" t="n">
         <v>0</v>
       </c>
       <c r="W169" t="n">
-        <v>254</v>
+        <v>274</v>
       </c>
       <c r="X169" t="n">
-        <v>269</v>
+        <v>249</v>
       </c>
       <c r="Y169" t="inlineStr">
         <is>
@@ -16646,12 +16667,12 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-05.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -16699,20 +16720,20 @@
         <v>75</v>
       </c>
       <c r="U170" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="V170" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W170" t="n">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="X170" t="n">
-        <v>357</v>
+        <v>348</v>
       </c>
       <c r="Y170" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="Z170" t="inlineStr"/>
@@ -16746,12 +16767,12 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-05.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -16846,12 +16867,12 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-05.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -17026,7 +17047,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -17080,7 +17101,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
@@ -17099,7 +17120,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -17148,17 +17169,17 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -17171,7 +17192,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-05-04.xlsx</t>
+          <t>TA 418 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -17220,12 +17241,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -17243,7 +17264,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -17278,7 +17299,7 @@
       <c r="I5" t="inlineStr">
         <is>
           <t>C3:Activity-&gt;activity_raw; C4:Quantity-&gt;quantity_loa; C5:unnamed_col_5-&gt;quantity_estimated_or_total; C7:unnamed_col_7-&gt;cumulative_last_month; C9:unnamed_col_9-&gt;plan_for_month; C10:Progress for the Month-&gt;progress_for_month; C11:unnamed_col_11-&gt;today_progress; C12:Cumulative Progress-&gt;cumulative_progress; C13:Balance Progress-&gt;balance_progress; C14:Gangs working 
-May-26-&gt;gangs_working; C15:2026-05-05 00:00:00 Remarks-&gt;remarks</t>
+May-26-&gt;gangs_working; C15:2026-05-10 00:00:00 Remarks-&gt;remarks</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -17297,7 +17318,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="O5" t="inlineStr"/>
@@ -17316,7 +17337,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-03.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -17365,12 +17386,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -17388,7 +17409,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-10.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -17441,7 +17462,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="O7" t="inlineStr"/>
@@ -17460,7 +17481,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TA 505 - DPR - 2026-04-17.xlsx</t>
+          <t>TA 505 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -17494,7 +17515,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>C2:PARTICULARS-&gt;activity_raw; C4:Total Qty-&gt;quantity_estimated_or_total; C5:Comp Till 2026-03-01 00:00:00-&gt;cumulative_last_month; C6:Balance as on 1st April-26-&gt;balance_progress; C7:April'26 Plan-&gt;plan_for_month; C8:Actual-&gt;progress_for_month; C10:Cumulative-&gt;cumulative_progress</t>
+          <t>C2:PARTICULARS-&gt;activity_raw; C4:Total Qty-&gt;quantity_estimated_or_total; C5:Comp Till 2026-04-01 00:00:00-&gt;cumulative_last_month; C6:Balance as on 1st May-26-&gt;balance_progress; C7:May'26 Plan-&gt;plan_for_month; C8:Actual-&gt;progress_for_month; C10:Cumulative-&gt;cumulative_progress</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
@@ -17509,7 +17530,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="O8" t="inlineStr"/>
@@ -17528,7 +17549,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-10.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -17581,7 +17602,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="O9" t="inlineStr"/>
@@ -17600,7 +17621,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TA 509 - DPR - 2026-01-17.xlsx</t>
+          <t>TA 509 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -17649,17 +17670,17 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>MATCH</t>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -17672,7 +17693,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -17721,7 +17742,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="O11" t="inlineStr"/>
@@ -17740,7 +17761,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -17792,7 +17813,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="O12" t="inlineStr"/>
@@ -17811,7 +17832,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -17861,12 +17882,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -17956,7 +17977,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -18010,7 +18031,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="O15" t="inlineStr"/>
@@ -18029,7 +18050,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -18083,7 +18104,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="O16" t="inlineStr"/>
@@ -18102,7 +18123,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-05.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -18153,12 +18174,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -18443,7 +18464,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -18461,7 +18482,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
@@ -18472,7 +18493,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Project Details; 765KV TA 414 VNTL; VNTL - KEC; Sheet5; Sheet3; Sheet1; DPR Sheet; FDN; FDN Completed; Erection ; Erection Completed ; Erection Compiled; Stringing Compiled; Sheet6; Sheet4; Sheet7; Stringing; Stringing Completed; Visual chart 1 ; Pile Fdn; Crossing; Sheet2; Soil Inv.; Survey Anx; Survey</t>
+          <t>Project Details; 765KV TA 414 VNTL; VNTL - KEC; Sheet5; Sheet3; Sheet1; DPR Sheet; FDN; FDN Completed; Erection ; Erection Completed ; Erection Compiled; Stringing; Stringing Completed; Stringing Compiled; Sheet6; Sheet4; Sheet7; Visual chart 1 ; Pile Fdn; Crossing; Sheet2; Soil Inv.; Survey Anx; Survey</t>
         </is>
       </c>
     </row>
@@ -18500,7 +18521,7 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-06.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -18518,17 +18539,17 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -18561,7 +18582,7 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-05-04.xlsx</t>
+          <t>TA 418 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -18579,12 +18600,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -18622,7 +18643,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -18640,7 +18661,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="K6" t="inlineStr"/>
@@ -18679,7 +18700,7 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-03.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -18697,12 +18718,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -18740,7 +18761,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-10.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -18758,7 +18779,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
@@ -18797,7 +18818,7 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>TA 505 - DPR - 2026-04-17.xlsx</t>
+          <t>TA 505 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -18815,7 +18836,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="K9" t="inlineStr"/>
@@ -18854,7 +18875,7 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-10.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-11.xlsx</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -18872,7 +18893,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="K10" t="inlineStr"/>
@@ -18911,7 +18932,7 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>TA 509 - DPR - 2026-01-17.xlsx</t>
+          <t>TA 509 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -18929,22 +18950,22 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>MATCH</t>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t xml:space="preserve">VC-765kV MKTL; SUMMARY; FOUNDATION; ERECTION; EARTHING; XING; SUPPLY; Sheet1; SURVEY SUMMARY; SURVEY STATUS ; Erection productivity; TS  25-10-25 </t>
+          <t>VC-765kV MKTL; SUMMARY; FDN pivot; Erc pivot; DPR; FOUNDATION; ERECTION; EARTHING; XING; SUPPLY; CST Gantry To AP 68 Common Poin; Sheet1; SURVEY SUMMARY; SURVEY STATUS ; Erection productivity</t>
         </is>
       </c>
     </row>
@@ -18972,7 +18993,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -18990,7 +19011,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
@@ -19029,7 +19050,7 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -19047,7 +19068,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
@@ -19058,7 +19079,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Concrete; Summary DPR; DPR S-F &amp; S-P (2); Summary; ERT; LS; Survey ; T.Marking; VC -SF; VC -SP; Ere S-P  ; Ere S-F ; FDN S-F; FDN S-P; T.Abstract; Supply.; Crossing status; Erection Compiled; Sheet5; Earthing S-P; Earthing S-F; Supply; ROW S-F; Proposal; Proposal .; ROW S-P; Master SP; Master SF; TS SP ; TS SF; Sheet4; Sheet2; Sheet1; Forest</t>
+          <t>Concrete; Summary DPR; DPR S-F &amp; S-P (2); Summary; ERT; LS; Survey ; T.Marking; VC -SF; VC -SP; Ere S-P  ; Ere S-F ; FDN S-F; FDN S-P; T.Abstract; Supply.; Crossing status; Erection Compiled; Sheet5; Earthing S-P; Supply; Earthing S-F; ROW S-F; Proposal; Proposal .; ROW S-P; Master SP; Master SF; TS SP ; TS SF; Sheet4; Sheet2; Sheet1; Forest</t>
         </is>
       </c>
     </row>
@@ -19086,7 +19107,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-05.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-09.xlsx</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -19104,12 +19125,12 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -19257,7 +19278,7 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -19275,7 +19296,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="K17" t="inlineStr"/>
@@ -19314,7 +19335,7 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-04.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -19332,7 +19353,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="K18" t="inlineStr"/>
@@ -19371,7 +19392,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-05.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-10.xlsx</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -19389,12 +19410,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -19404,7 +19425,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>TB401 DPR.....; Eng.; Fdn (Pkg -G Section -I); Sheet2; Sheet3; Sheet4; Sheet5; ROW; Sheet13 (2); TB-605; Sheet19; Sheet16; Sheet14; Sheet12; Sheet13; Sheet15; TB401 DPR; Survey-Summary; Sheet6; Approved Survey; Approved CS J-S Line; Approved CS K-S Line; Foundation JS-Line -Jammu; Sheet10; Erection -Jammu; Vertical Chart -JS Line Jammu ; Sheet17; Erection -SK; Sheet7; Sheet8; Foundation -LILO; Erection-Punjab; Vertical Chart -JS Line Punjab; Foundation -JS Line- Punjab; Sheet9; ROW Front vs Progress; Hindrance; Foundation -KS Line; Manpower; Sum; Sheet18; JS-Supply Stubs; JS Supply Towers; SK Supply Stubs; SK Supply Towers; Sheet11; Planned Vs Actual -FDN; Supply Status; Material Status-Jammu-Punjab; Material Status-Punjab; Earthing (PKG-F); Earthing (PKG-G); Revetment Pkg-G;  Benching Status-F;  Benching Status-G; Earthing Pkg -G Ist section; Earthing balance; Tack Welding - PKG-G; Tack Welding - PKG-F; Painting - PKG-G; Painting - PKG-F; Eretion - PKG-G; Eretion - PKG-F; Sheet1; JMC 27.9.23; Jumpering-G; Insulator Hoisting - F; Insulator Hoisting - G; Jumpering-F; Stringing - PKG-F; Stringing - PKG-G; OPGW PKG-G; OPGW PKG-F; Crossing; Clear locs shared by client</t>
+          <t>TB401 DPR.....; Eng.; Fdn (Pkg -G Section -I); Sheet2; Sheet3; Sheet4; Sheet5; ROW; Sheet13 (2); TB-605; Sheet19; Sheet16; Sheet14; Sheet12; Sheet13; Sheet15; TB401 DPR; Survey-Summary; Sheet6; Approved Survey; Approved CS J-S Line; Approved CS K-S Line; Foundation JS-Line -Jammu; Sheet10; Erection -Jammu; Vertical Chart -JS Line Jammu ; Sheet17; Erection -SK; Sheet7; Sheet8; LILO; Erection-Punjab; Vertical Chart -JS Line Punjab; Foundation -JS Line- Punjab; Sheet9; ROW Front vs Progress; Hindrance; Foundation -KS Line; Manpower; Sum; Sheet18; JS-Supply Stubs; JS Supply Towers; SK Supply Stubs; SK Supply Towers; Sheet11; Planned Vs Actual -FDN; Supply Status; Material Status-Jammu-Punjab; Material Status-Punjab; Earthing (PKG-F); Earthing (PKG-G); Revetment Pkg-G;  Benching Status-F;  Benching Status-G; Earthing Pkg -G Ist section; Earthing balance; Tack Welding - PKG-G; Tack Welding - PKG-F; Painting - PKG-G; Painting - PKG-F; Eretion - PKG-G; Eretion - PKG-F; Sheet1; JMC 27.9.23; Jumpering-G; Insulator Hoisting - F; Insulator Hoisting - G; Jumpering-F; Stringing - PKG-F; Stringing - PKG-G; OPGW PKG-G; OPGW PKG-F; Crossing; Clear locs shared by client</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-21 11:45:02
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -597,12 +597,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -698,12 +698,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -799,12 +799,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -900,12 +900,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1001,12 +1001,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1102,12 +1102,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1203,12 +1203,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1306,12 +1306,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1409,12 +1409,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1512,12 +1512,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1611,12 +1611,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1710,12 +1710,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1766,16 +1766,16 @@
         <v>40</v>
       </c>
       <c r="V13" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="W13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X13" t="n">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="Y13" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
@@ -1817,12 +1817,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1924,12 +1924,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2027,12 +2027,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2126,12 +2126,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -6612,12 +6612,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -6703,12 +6703,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -6796,12 +6796,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -6891,12 +6891,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -6984,12 +6984,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -7077,12 +7077,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -7756,12 +7756,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -7847,12 +7847,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -7938,12 +7938,12 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -8033,12 +8033,12 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -8128,12 +8128,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -8223,12 +8223,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -18079,12 +18079,12 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -18182,12 +18182,12 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -18285,12 +18285,12 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -18388,12 +18388,12 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -18491,12 +18491,12 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -18549,9 +18549,7 @@
       <c r="V185" t="n">
         <v>15</v>
       </c>
-      <c r="W185" t="n">
-        <v>1</v>
-      </c>
+      <c r="W185" t="inlineStr"/>
       <c r="X185" t="n">
         <v>304</v>
       </c>
@@ -18560,12 +18558,12 @@
       </c>
       <c r="Z185" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="AA185" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>40.0</t>
         </is>
       </c>
     </row>
@@ -18602,12 +18600,12 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -18703,12 +18701,12 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -18761,9 +18759,7 @@
       <c r="V187" t="n">
         <v>16</v>
       </c>
-      <c r="W187" t="n">
-        <v>2</v>
-      </c>
+      <c r="W187" t="inlineStr"/>
       <c r="X187" t="n">
         <v>210</v>
       </c>
@@ -18772,12 +18768,12 @@
       </c>
       <c r="Z187" t="inlineStr">
         <is>
-          <t>7.0</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="AA187" t="inlineStr">
         <is>
-          <t>144.0</t>
+          <t>141.0</t>
         </is>
       </c>
     </row>
@@ -18814,12 +18810,12 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -18921,12 +18917,12 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -19006,12 +19002,12 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -19115,12 +19111,12 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -19216,12 +19212,12 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -19309,12 +19305,12 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -19404,12 +19400,12 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -19499,12 +19495,12 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -19602,12 +19598,12 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -19705,12 +19701,12 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -19808,12 +19804,12 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -19911,12 +19907,12 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -19970,7 +19966,7 @@
         <v>8</v>
       </c>
       <c r="W199" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X199" t="n">
         <v>30</v>
@@ -19980,12 +19976,12 @@
       </c>
       <c r="Z199" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="AA199" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>45.0</t>
         </is>
       </c>
     </row>
@@ -20022,12 +20018,12 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -20125,12 +20121,12 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -20232,12 +20228,12 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -20327,12 +20323,12 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -20414,12 +20410,12 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -20511,12 +20507,12 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -20608,12 +20604,12 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -25127,7 +25123,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -25183,7 +25179,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -25568,7 +25564,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -25621,7 +25617,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O8" t="inlineStr"/>
@@ -25708,7 +25704,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -25761,7 +25757,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O10" t="inlineStr"/>
@@ -26281,7 +26277,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -26335,7 +26331,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="O18" t="inlineStr"/>
@@ -26354,7 +26350,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -26408,7 +26404,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="O19" t="inlineStr"/>
@@ -26795,7 +26791,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -26813,7 +26809,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -27153,7 +27149,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -27171,7 +27167,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
@@ -27267,7 +27263,7 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -27285,7 +27281,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K10" t="inlineStr"/>
@@ -27849,7 +27845,7 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -27867,7 +27863,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
@@ -27878,7 +27874,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>400kV Summery; Check Survey ; Check Survey Status; Check Survey; Sheet8; Sheet2; Project Details; Statutory Clearence;  Crossing Proposal; Sheet1; VC 51-96; VC; ROW; June; Foundation; Royalty; Sheet14; Sheet7; Erection ; Completion date; Erection Compiled ; Earthing; Final Check In And Tack Welding; Stringing Compiled ; Soil Investigation; Sheet9; VC ; Sheet6; VC 51-121; Sheet5; Sheet3; Tower Schedule; Visual Chart; L2 Vs Actual Progress Chart; L2 Vs Actual Progress Chart (2); Sheet4</t>
+          <t>400kV Summery; Check Survey ; Check Survey Status; Check Survey; Sheet8; Sheet2; Project Details; Statutory Clearence;  Crossing Proposal; Sheet1; VC 51-96; VC; ROW; June; Foundation; Royalty; Sheet14; Sheet7; Erection ; Completion date; Erection Compiled ; Earthing; Final Check In And Tack Welding; Sheet10; Stringing Compiled ; Soil Investigation; Sheet9; VC ; Sheet6; VC 51-121; Sheet5; Sheet3; Tower Schedule; Visual Chart; L2 Vs Actual Progress Chart; L2 Vs Actual Progress Chart (2); Sheet4</t>
         </is>
       </c>
     </row>
@@ -27906,7 +27902,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-19.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -27924,7 +27920,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-21 12:16:27
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -5614,12 +5614,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -5715,12 +5715,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5814,12 +5814,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -5915,12 +5915,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -5973,14 +5973,14 @@
         <v>40</v>
       </c>
       <c r="V56" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="W56" t="inlineStr"/>
       <c r="X56" t="n">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="Y56" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="Z56" t="inlineStr">
         <is>
@@ -6018,12 +6018,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="Z57" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="AA57" t="inlineStr"/>
@@ -6121,12 +6121,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -6228,12 +6228,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -6288,9 +6288,7 @@
       <c r="V59" t="n">
         <v>6.21075</v>
       </c>
-      <c r="W59" t="n">
-        <v>2.262</v>
-      </c>
+      <c r="W59" t="inlineStr"/>
       <c r="X59" t="n">
         <v>113.36075</v>
       </c>
@@ -6329,12 +6327,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -6426,12 +6424,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -6519,12 +6517,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -25492,7 +25490,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -25541,17 +25539,17 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>MATCH</t>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -27088,7 +27086,7 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -27106,22 +27104,22 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>MATCH</t>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Project Details; Master Sheet; ProGress Sheet ; Erection Compiled ; Stringing Compiled ; Erection Productivity ; Visual Chart ; Stubs and Towers ; SuPPLY ; X-ing Details ; Tack Welding ; Tower Accessories ; Tower Tightening ; Hardwares &amp; Tower Accessories </t>
+          <t>Project Details; Master Sheet; ProGress Sheet ; Erection Compiled ; Stringing Compiled ; Erection Productivity ; Visual Chart ; Stubs and Towers ; SuPPLY ; X-ing Details ; Tack Welding ; Tower Accessories ; Tower Tightening ; Hardwares &amp; Tower Accessories ; Sheet1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-21 16:19:57
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -4286,12 +4286,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -4383,12 +4383,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -4480,12 +4480,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -4573,12 +4573,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4666,12 +4666,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4759,12 +4759,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4815,14 +4815,14 @@
         <v>45</v>
       </c>
       <c r="V44" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="W44" t="inlineStr"/>
       <c r="X44" t="n">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="Y44" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="Z44" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>37/0, 38/2, 52/1, 52/2, 54/0,  59/0, 66/0, 67/0, 69/0, 70/0,72/0, 73/0, 75/0, 76/0, 76/1, 82/0, 87/1, 95A/0, 96/0</t>
+          <t>37/0, 38/2, 39/0, 52/1, 52/2, 54/0,  59/0, 65/2, 66/0, 68/0, 70/0,72/0, 73/0, 75/0, 76/0, 76/1, 82/0, 87/1, 95A/0, 96/0</t>
         </is>
       </c>
     </row>
@@ -4864,12 +4864,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4961,12 +4961,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -5017,14 +5017,14 @@
         <v>40</v>
       </c>
       <c r="V46" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W46" t="inlineStr"/>
       <c r="X46" t="n">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="Y46" t="n">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Z46" t="inlineStr">
         <is>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>13/0,  14/1, 40/8, 42/0 , 62/0,  64/2, 64/3, 81/0</t>
+          <t>13/0, 15/0, 14/1, 32/0, 42/0 , 61/0,  62/0,  64/2, 64/3, 81/0</t>
         </is>
       </c>
     </row>
@@ -5066,12 +5066,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -5165,12 +5165,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -5254,12 +5254,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -5347,12 +5347,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -5440,12 +5440,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -5533,12 +5533,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -25417,7 +25417,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -25452,7 +25452,7 @@
       <c r="I6" t="inlineStr">
         <is>
           <t>C3:Activity-&gt;activity_raw; C4:Quantity-&gt;quantity_loa; C5:unnamed_col_5-&gt;quantity_estimated_or_total; C7:unnamed_col_7-&gt;cumulative_last_month; C9:unnamed_col_9-&gt;plan_for_month; C10:Progress for the Month-&gt;progress_for_month; C11:unnamed_col_11-&gt;today_progress; C12:Cumulative Progress-&gt;cumulative_progress; C13:Balance Progress-&gt;balance_progress; C14:Gangs working 
-May-26-&gt;gangs_working; C15:2026-05-18 00:00:00 Remarks-&gt;remarks</t>
+May-26-&gt;gangs_working; C15:2026-05-20 00:00:00 Remarks-&gt;remarks</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -25471,7 +25471,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -27029,7 +27029,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -27047,7 +27047,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="K6" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-22 10:45:01
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -597,12 +597,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -698,12 +698,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -799,12 +799,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -900,12 +900,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1001,12 +1001,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1102,12 +1102,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1203,12 +1203,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1306,12 +1306,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1409,12 +1409,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1512,12 +1512,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1611,12 +1611,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1710,12 +1710,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1766,16 +1766,16 @@
         <v>40</v>
       </c>
       <c r="V13" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="W13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X13" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="Y13" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
@@ -1817,12 +1817,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1924,12 +1924,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2027,12 +2027,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2126,12 +2126,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -3476,12 +3476,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-17.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3577,12 +3577,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-17.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3678,12 +3678,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-17.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3779,12 +3779,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-17.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3833,20 +3833,20 @@
         <v>8.4</v>
       </c>
       <c r="V34" t="n">
-        <v>3.374</v>
+        <v>4.051</v>
       </c>
       <c r="W34" t="n">
         <v>0</v>
       </c>
       <c r="X34" t="n">
-        <v>110.097</v>
+        <v>110.774</v>
       </c>
       <c r="Y34" t="n">
-        <v>5.036999999999992</v>
+        <v>4.359999999999985</v>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AA34" t="inlineStr"/>
@@ -5614,12 +5614,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -5715,12 +5715,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5814,12 +5814,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -5915,12 +5915,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -6018,12 +6018,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -6121,12 +6121,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -6195,7 +6195,7 @@
       </c>
       <c r="AA58" t="inlineStr">
         <is>
-          <t>35/0 - 36/0 - Conductor payingout under progreess +34/2 -35/0 - Conductor passing under progress + 33/0 -34/0 - WIP</t>
+          <t>35/0 - 36/0 - Conductor payingout under progreess +34/2 -35/0 - Conductor passing under progress + 33/0 -34/0 - Insualtor Hosting under progress</t>
         </is>
       </c>
     </row>
@@ -6228,12 +6228,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -6327,12 +6327,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -6424,12 +6424,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -6517,12 +6517,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -8700,12 +8700,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -8797,12 +8797,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -8894,12 +8894,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -8991,12 +8991,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -9088,12 +9088,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -9185,12 +9185,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -9288,12 +9288,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -9385,12 +9385,12 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -9443,14 +9443,16 @@
         <v>18</v>
       </c>
       <c r="V92" t="n">
-        <v>6</v>
-      </c>
-      <c r="W92" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="W92" t="n">
+        <v>1</v>
+      </c>
       <c r="X92" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Y92" t="n">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="Z92" t="inlineStr">
         <is>
@@ -9488,12 +9490,12 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -9585,12 +9587,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -9682,12 +9684,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -9779,12 +9781,12 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -9876,12 +9878,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -9973,12 +9975,12 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -10074,12 +10076,12 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -10175,12 +10177,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -10276,12 +10278,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -10377,12 +10379,12 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -10435,7 +10437,7 @@
         <v>272</v>
       </c>
       <c r="V102" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W102" t="n">
         <v>25</v>
@@ -10444,7 +10446,7 @@
         <v>1</v>
       </c>
       <c r="Y102" t="n">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="Z102" t="inlineStr"/>
       <c r="AA102" t="inlineStr"/>
@@ -10478,12 +10480,12 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -10536,16 +10538,16 @@
         <v>272</v>
       </c>
       <c r="V103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W103" t="n">
         <v>25</v>
       </c>
       <c r="X103" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y103" t="n">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="Z103" t="inlineStr">
         <is>
@@ -10583,12 +10585,12 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -10676,12 +10678,12 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -10781,12 +10783,12 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -10839,14 +10841,14 @@
         <v>0</v>
       </c>
       <c r="V106" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="W106" t="inlineStr"/>
       <c r="X106" t="n">
         <v>1</v>
       </c>
       <c r="Y106" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Z106" t="inlineStr"/>
       <c r="AA106" t="inlineStr"/>
@@ -10880,12 +10882,12 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -10979,12 +10981,12 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -11078,12 +11080,12 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -11177,12 +11179,12 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -11276,12 +11278,12 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -11373,12 +11375,12 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -11470,12 +11472,12 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -11565,12 +11567,12 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -11660,12 +11662,12 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -11755,12 +11757,12 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -11854,12 +11856,12 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -11910,16 +11912,16 @@
         <v>350</v>
       </c>
       <c r="V117" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="W117" t="n">
         <v>1</v>
       </c>
       <c r="X117" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="Y117" t="n">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="Z117" t="inlineStr">
         <is>
@@ -11928,10 +11930,9 @@
       </c>
       <c r="AA117" t="inlineStr">
         <is>
-          <t>Loc-55/7-Casting WIP
-Loc-64/5-Casting  compl
-Loc-64/3-PCC WIP
-Loc-74/9-Pit Marking done</t>
+          <t>Loc-51/3-Casting WIP
+Loc-64/3-Casting Compl
+Loc-74/9-Excavation compl</t>
         </is>
       </c>
     </row>
@@ -11964,12 +11965,12 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -12059,12 +12060,12 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -12131,7 +12132,7 @@
       </c>
       <c r="AA119" t="inlineStr">
         <is>
-          <t>51/4-Tower erection WIP</t>
+          <t>51/4-Tower erection WIP(3rd Section compl)</t>
         </is>
       </c>
     </row>
@@ -12164,12 +12165,12 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -12259,12 +12260,12 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -12352,12 +12353,12 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -12445,12 +12446,12 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -12538,12 +12539,12 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -12633,12 +12634,12 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -12728,12 +12729,12 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -12823,12 +12824,12 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -12918,12 +12919,12 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -13013,12 +13014,12 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -13108,12 +13109,12 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -13207,12 +13208,12 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -13281,7 +13282,7 @@
       </c>
       <c r="AA131" t="inlineStr">
         <is>
-          <t>Loc-28/1-Steel Binding U/P</t>
+          <t>Loc-28/1-Casting  U/P</t>
         </is>
       </c>
     </row>
@@ -13314,12 +13315,12 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -13411,12 +13412,12 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -13506,12 +13507,12 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -13599,12 +13600,12 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -13690,12 +13691,12 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -13779,12 +13780,12 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -13868,12 +13869,12 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -13959,12 +13960,12 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -14016,7 +14017,7 @@
         <v>7</v>
       </c>
       <c r="W139" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X139" t="n">
         <v>120</v>
@@ -14060,12 +14061,12 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -14117,7 +14118,7 @@
         <v>9</v>
       </c>
       <c r="W140" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X140" t="n">
         <v>98</v>
@@ -14157,12 +14158,12 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -14258,12 +14259,12 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -14355,12 +14356,12 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -14452,12 +14453,12 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -14549,12 +14550,12 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -14636,12 +14637,12 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -14723,12 +14724,12 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -14810,12 +14811,12 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -14897,12 +14898,12 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -14978,12 +14979,12 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -15026,13 +15027,13 @@
         <v>186.3</v>
       </c>
       <c r="R150" t="n">
-        <v>184.963</v>
+        <v>185.149</v>
       </c>
       <c r="S150" t="n">
-        <v>184.963</v>
+        <v>185.149</v>
       </c>
       <c r="T150" t="n">
-        <v>184.963</v>
+        <v>185.149</v>
       </c>
       <c r="U150" t="n">
         <v>0</v>
@@ -15040,7 +15041,7 @@
       <c r="V150" t="inlineStr"/>
       <c r="W150" t="inlineStr"/>
       <c r="X150" t="n">
-        <v>184.963</v>
+        <v>185.149</v>
       </c>
       <c r="Y150" t="n">
         <v>0</v>
@@ -15077,12 +15078,12 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -15174,12 +15175,12 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -15259,12 +15260,12 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -15344,12 +15345,12 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -15404,14 +15405,16 @@
         <v>35</v>
       </c>
       <c r="V154" t="n">
-        <v>7</v>
-      </c>
-      <c r="W154" t="inlineStr"/>
+        <v>9</v>
+      </c>
+      <c r="W154" t="n">
+        <v>1</v>
+      </c>
       <c r="X154" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="Y154" t="n">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="Z154" t="inlineStr">
         <is>
@@ -15449,12 +15452,12 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -15550,12 +15553,12 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -15639,12 +15642,12 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -15728,12 +15731,12 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -15823,12 +15826,12 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -15920,12 +15923,12 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -15980,16 +15983,16 @@
         <v>40</v>
       </c>
       <c r="V160" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="W160" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X160" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="Y160" t="n">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="Z160" t="inlineStr">
         <is>
@@ -16027,12 +16030,12 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -16132,12 +16135,12 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -16233,12 +16236,12 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -16338,12 +16341,12 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -16439,12 +16442,12 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -16497,16 +16500,16 @@
         <v>4</v>
       </c>
       <c r="V165" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W165" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X165" t="n">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="Y165" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z165" t="inlineStr">
         <is>
@@ -16515,7 +16518,7 @@
       </c>
       <c r="AA165" t="inlineStr">
         <is>
-          <t>34/0 erection under progress</t>
+          <t>34/0 erection completed</t>
         </is>
       </c>
     </row>
@@ -16548,12 +16551,12 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -16653,12 +16656,12 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -16740,12 +16743,12 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -16845,12 +16848,12 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -16946,12 +16949,12 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -17051,12 +17054,12 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -17150,12 +17153,12 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -17249,12 +17252,12 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -17358,12 +17361,12 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -17463,12 +17466,12 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -17568,12 +17571,12 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -17673,12 +17676,12 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -17758,12 +17761,12 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -17832,11 +17835,7 @@
           <t>1.0</t>
         </is>
       </c>
-      <c r="AA178" t="inlineStr">
-        <is>
-          <t>10/0, 11/0 Jumper work done</t>
-        </is>
-      </c>
+      <c r="AA178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -17867,12 +17866,12 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -17968,12 +17967,12 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -20695,12 +20694,12 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -20794,12 +20793,12 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -20848,20 +20847,20 @@
         <v>72</v>
       </c>
       <c r="V208" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="W208" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X208" t="n">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="Y208" t="n">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="Z208" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>35</t>
         </is>
       </c>
       <c r="AA208" t="inlineStr"/>
@@ -20895,12 +20894,12 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -20996,12 +20995,12 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
@@ -21050,16 +21049,16 @@
         <v>75</v>
       </c>
       <c r="V210" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="W210" t="n">
         <v>2</v>
       </c>
       <c r="X210" t="n">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="Y210" t="n">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="Z210" t="inlineStr">
         <is>
@@ -21097,12 +21096,12 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
@@ -21198,12 +21197,12 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
@@ -25121,7 +25120,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -25177,7 +25176,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -25273,7 +25272,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-17.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -25322,17 +25321,17 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -25490,7 +25489,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -25539,7 +25538,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -25549,7 +25548,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -25846,7 +25845,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -25884,11 +25883,7 @@
 till last Month (Mar'26)-&gt;cumulative_last_month; C6:L3 Plan for the month (April'26 )-&gt;plan_for_month; C7:Today's Progress-&gt;today_progress; C8:Progress in this month-&gt;progress_for_month; C9:Cumm. Progress till date-&gt;cumulative_progress; C10:Cumm. Balance-&gt;balance_progress; C12:No of Gangs-&gt;gangs_working; C13:Remark-&gt;remarks</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>XML scrub fallback used for sheet 'AOTL - KEC'</t>
-        </is>
-      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="n">
         <v>1</v>
       </c>
@@ -25900,7 +25895,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O12" t="inlineStr"/>
@@ -25919,7 +25914,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -25968,7 +25963,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O13" t="inlineStr"/>
@@ -25987,7 +25982,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -26039,7 +26034,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O14" t="inlineStr"/>
@@ -26058,7 +26053,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -26108,12 +26103,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -26131,7 +26126,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -26180,12 +26175,12 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -26203,7 +26198,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -26252,12 +26247,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -26421,7 +26416,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -26472,12 +26467,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -26789,7 +26784,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -26807,7 +26802,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -26907,7 +26902,7 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-17.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -26925,17 +26920,17 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -27086,7 +27081,7 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -27104,7 +27099,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -27114,7 +27109,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -27379,7 +27374,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -27397,7 +27392,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
@@ -27408,7 +27403,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>765KV TA 414 VNTL; 765KV ASOTL; Project Details; AOTL - KEC; DPR Sheet; Sheet5; Sheet3; Sheet1; Survey Anx; Soil Inv.; Survey; FDN; Erection ; Erection Compiled ; Visual chart 1 ; Pile Foundation; Sheet6; Sheet4; Sheet7; Tack welding; Stringing Compiled; String; Crossing; Tree Enumeration; Sheet2</t>
+          <t>765KV TA 414 VNTL; 765KV ASOTL; Project Details; AOTL - KEC; DPR Sheet; Sheet5; Sheet3; Sheet1; Survey Anx; Soil Inv.; Survey; FDN; Erection ; Visual chart 1 ; Pile Foundation; Sheet6; Sheet4; Sheet7; Tack welding; Stringing Compiled; String; Crossing; Tree Enumeration; Sheet2</t>
         </is>
       </c>
     </row>
@@ -27436,7 +27431,7 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -27454,7 +27449,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
@@ -27493,7 +27488,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-19.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -27511,7 +27506,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
@@ -27611,7 +27606,7 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -27629,12 +27624,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -27672,7 +27667,7 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-18.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -27690,12 +27685,12 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -27705,7 +27700,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>DPR-KEC; Survey details; Visual Chart ; Detail Survey; Check Survey ; FDN; Composite-Survey(05-04-2026); Erection; Earthing; WIP; statuary clearance; statuary clearance (2); Supply Status</t>
+          <t>DPR-KEC; Survey details; FDN; Erection; Visual Chart ; Detail Survey; Check Survey ; Composite-Survey(05-04-2026); Earthing; WIP; statuary clearance; statuary clearance (2); Supply Status</t>
         </is>
       </c>
     </row>
@@ -27782,7 +27777,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -27800,12 +27795,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -27957,7 +27952,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -27975,12 +27970,12 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -27990,7 +27985,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>TB401 DPR.....; Eng.; Fdn (Pkg -G Section -I); Sheet2; Sheet3; Sheet4; Sheet5; ROW; Sheet13 (2); TB-605; Sheet19; Sheet16; Sheet14; Sheet12; Sheet13; Sheet15; TB401 DPR; Survey-Summary; Sheet6; Approved Survey; Approved CS J-S Line; Approved CS K-S Line; Foundation JS-Line -Jammu; Sheet10; Erection -Jammu; Vertical Chart -JS Line Jammu ; Sheet17; Erection -SK; Sheet7; Sheet8; LILO; Erection-Punjab; Vertical Chart -JS Line Punjab; Foundation -JS Line- Punjab; Sheet9; ROW Front vs Progress; Hindrance; Foundation -KS Line; Manpower; Sum; Sheet18; JS-Supply Stubs; JS Supply Towers; SK Supply Stubs; SK Supply Towers; Sheet11; Planned Vs Actual -FDN; Supply Status; Material Status-Jammu-Punjab; Material Status-Punjab; Earthing (PKG-F); Earthing (PKG-G); Revetment Pkg-G;  Benching Status-F;  Benching Status-G; Earthing Pkg -G Ist section; Earthing balance; Tack Welding - PKG-G; Tack Welding - PKG-F; Painting - PKG-G; Painting - PKG-F; Eretion - PKG-G; Eretion - PKG-F; Sheet1; JMC 27.9.23; Jumpering-G; Insulator Hoisting - F; Insulator Hoisting - G; Jumpering-F; Stringing - PKG-F; Stringing - PKG-G; OPGW PKG-G; OPGW PKG-F; Crossing; Clear locs shared by client</t>
+          <t>TB401 DPR.....; Eng.; Fdn (Pkg -G Section -I); Sheet2; Sheet3; Sheet4; Sheet5; ROW; Sheet13 (2); TB-605; Sheet19; Sheet16; Sheet14; Sheet12; Sheet13; Sheet15; TB401 DPR; Survey-Summary; Sheet6; Approved Survey; Approved CS J-S Line; Approved CS K-S Line; Foundation JS-Line -Jammu; Sheet10; Erection -Jammu; Vertical Chart -JS Line Jammu ; Sheet17; Erection -SK; Sheet7; Sheet8; LILO; Erection-Punjab; Vertical Chart -JS Line Punjab; Foundation -JS Line- Punjab; Sheet9; ROW Front vs Progress; Hindrance; Foundation -KS Line; Manpower; Stubs JS; Stubs SK; Towers JS; Towers SK; Sum; Sheet18; JS-Supply Stubs; JS Supply Towers; SK Supply Stubs; SK Supply Towers; Sheet11; Planned Vs Actual -FDN; Supply Status; Material Status-Jammu-Punjab; Material Status-Punjab; Earthing (PKG-F); Earthing (PKG-G); Revetment Pkg-G;  Benching Status-F;  Benching Status-G; Earthing Pkg -G Ist section; Earthing balance; Tack Welding - PKG-G; Tack Welding - PKG-F; Painting - PKG-G; Painting - PKG-F; Eretion - PKG-G; Eretion - PKG-F; Sheet1; JMC 27.9.23; Jumpering-G; Insulator Hoisting - F; Insulator Hoisting - G; Jumpering-F; Stringing - PKG-F; Stringing - PKG-G; OPGW PKG-G; OPGW PKG-F; Crossing; Clear locs shared by client</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-22 12:16:59
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -4286,12 +4286,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -4383,12 +4383,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -4480,12 +4480,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -4573,12 +4573,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4666,12 +4666,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4759,12 +4759,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4826,12 +4826,12 @@
       </c>
       <c r="Z44" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>37/0, 38/2, 39/0, 52/1, 52/2, 54/0,  59/0, 65/2, 66/0, 68/0, 70/0,72/0, 73/0, 75/0, 76/0, 76/1, 82/0, 87/1, 95A/0, 96/0</t>
+          <t>37/0, 38/2, 39/0, 47/0, 52/1, 52/2, 54/0,  59/0, 65/2, 66/0, 68/0, 70/0,72/0, 73/0, 75/0, 76/0, 76/1, 82/0, 87/1, 95A/0, 96/0</t>
         </is>
       </c>
     </row>
@@ -4864,12 +4864,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4961,12 +4961,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -5066,12 +5066,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -5165,12 +5165,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -5254,12 +5254,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -5347,12 +5347,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -5440,12 +5440,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -5533,12 +5533,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -18076,12 +18076,12 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -18179,12 +18179,12 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -18282,12 +18282,12 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -18385,12 +18385,12 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -18488,12 +18488,12 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -18560,7 +18560,7 @@
       </c>
       <c r="AA185" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>35.0</t>
         </is>
       </c>
     </row>
@@ -18597,12 +18597,12 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -18698,12 +18698,12 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -18807,12 +18807,12 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -18914,12 +18914,12 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -18999,12 +18999,12 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -19057,7 +19057,9 @@
       <c r="V190" t="n">
         <v>3.712</v>
       </c>
-      <c r="W190" t="inlineStr"/>
+      <c r="W190" t="n">
+        <v>0.165</v>
+      </c>
       <c r="X190" t="n">
         <v>21.195</v>
       </c>
@@ -19108,12 +19110,12 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -19209,12 +19211,12 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -19302,12 +19304,12 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -19397,12 +19399,12 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -19492,12 +19494,12 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -19595,12 +19597,12 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -19698,12 +19700,12 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -19801,12 +19803,12 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -19904,12 +19906,12 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -19960,16 +19962,16 @@
         <v>11</v>
       </c>
       <c r="V199" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W199" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X199" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Y199" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="Z199" t="inlineStr">
         <is>
@@ -19978,7 +19980,7 @@
       </c>
       <c r="AA199" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>50.0</t>
         </is>
       </c>
     </row>
@@ -20015,12 +20017,12 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -20118,12 +20120,12 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -20225,12 +20227,12 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -20320,12 +20322,12 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -20407,12 +20409,12 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -20504,12 +20506,12 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -20601,12 +20603,12 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -25416,7 +25418,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -25451,7 +25453,7 @@
       <c r="I6" t="inlineStr">
         <is>
           <t>C3:Activity-&gt;activity_raw; C4:Quantity-&gt;quantity_loa; C5:unnamed_col_5-&gt;quantity_estimated_or_total; C7:unnamed_col_7-&gt;cumulative_last_month; C9:unnamed_col_9-&gt;plan_for_month; C10:Progress for the Month-&gt;progress_for_month; C11:unnamed_col_11-&gt;today_progress; C12:Cumulative Progress-&gt;cumulative_progress; C13:Balance Progress-&gt;balance_progress; C14:Gangs working 
-May-26-&gt;gangs_working; C15:2026-05-20 00:00:00 Remarks-&gt;remarks</t>
+May-26-&gt;gangs_working; C15:2026-05-21 00:00:00 Remarks-&gt;remarks</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -25470,7 +25472,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -26270,7 +26272,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -26324,7 +26326,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O18" t="inlineStr"/>
@@ -26343,7 +26345,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -26397,7 +26399,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O19" t="inlineStr"/>
@@ -27024,7 +27026,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-20.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -27042,7 +27044,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K6" t="inlineStr"/>
@@ -27838,7 +27840,7 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -27856,7 +27858,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
@@ -27895,7 +27897,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-20.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -27913,7 +27915,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-25 10:43:46
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -597,12 +597,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -698,12 +698,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -799,12 +799,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -900,12 +900,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1001,12 +1001,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1102,12 +1102,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1203,12 +1203,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1306,12 +1306,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1409,12 +1409,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1512,12 +1512,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1611,12 +1611,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1710,12 +1710,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1766,16 +1766,16 @@
         <v>40</v>
       </c>
       <c r="V13" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="W13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X13" t="n">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="Y13" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
@@ -1817,12 +1817,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1924,12 +1924,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1994,7 +1994,7 @@
       <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>G_2:- SK infra  (MP 60)</t>
+          <t>_2:- SK infra  (MP 45)</t>
         </is>
       </c>
     </row>
@@ -2027,12 +2027,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2126,12 +2126,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2225,12 +2225,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2316,12 +2316,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2407,12 +2407,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2498,12 +2498,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2589,12 +2589,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2643,16 +2643,14 @@
         <v>34</v>
       </c>
       <c r="V22" t="n">
-        <v>12</v>
-      </c>
-      <c r="W22" t="n">
-        <v>2</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="W22" t="inlineStr"/>
       <c r="X22" t="n">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="Y22" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr"/>
@@ -2686,12 +2684,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2740,16 +2738,14 @@
         <v>34</v>
       </c>
       <c r="V23" t="n">
-        <v>12</v>
-      </c>
-      <c r="W23" t="n">
-        <v>2</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="W23" t="inlineStr"/>
       <c r="X23" t="n">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="Y23" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -2787,12 +2783,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2841,7 +2837,7 @@
         <v>34</v>
       </c>
       <c r="V24" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="W24" t="inlineStr"/>
       <c r="X24" t="n">
@@ -2882,12 +2878,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2936,20 +2932,20 @@
         <v>55</v>
       </c>
       <c r="V25" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="W25" t="n">
         <v>1</v>
       </c>
       <c r="X25" t="n">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="Y25" t="n">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>14.0</t>
         </is>
       </c>
       <c r="AA25" t="inlineStr">
@@ -2987,12 +2983,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -3041,16 +3037,14 @@
         <v>55</v>
       </c>
       <c r="V26" t="n">
-        <v>14</v>
-      </c>
-      <c r="W26" t="n">
-        <v>2</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="W26" t="inlineStr"/>
       <c r="X26" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="Y26" t="n">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
@@ -3088,12 +3082,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -3142,16 +3136,14 @@
         <v>20</v>
       </c>
       <c r="V27" t="n">
-        <v>3.768</v>
-      </c>
-      <c r="W27" t="n">
-        <v>0.228</v>
-      </c>
+        <v>6.052</v>
+      </c>
+      <c r="W27" t="inlineStr"/>
       <c r="X27" t="n">
-        <v>10.396</v>
+        <v>12.68</v>
       </c>
       <c r="Y27" t="n">
-        <v>117.403</v>
+        <v>115.119</v>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
@@ -3189,12 +3181,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -3245,9 +3237,7 @@
       <c r="V28" t="n">
         <v>6.401</v>
       </c>
-      <c r="W28" t="n">
-        <v>0.228</v>
-      </c>
+      <c r="W28" t="inlineStr"/>
       <c r="X28" t="n">
         <v>18.097</v>
       </c>
@@ -3286,12 +3276,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3340,16 +3330,14 @@
         <v>20</v>
       </c>
       <c r="V29" t="n">
-        <v>3.768</v>
-      </c>
-      <c r="W29" t="n">
-        <v>0.228</v>
-      </c>
+        <v>6.052</v>
+      </c>
+      <c r="W29" t="inlineStr"/>
       <c r="X29" t="n">
-        <v>10.396</v>
+        <v>12.68</v>
       </c>
       <c r="Y29" t="n">
-        <v>117.403</v>
+        <v>115.119</v>
       </c>
       <c r="Z29" t="inlineStr"/>
       <c r="AA29" t="inlineStr"/>
@@ -3383,12 +3371,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -3476,12 +3464,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3577,12 +3565,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3678,12 +3666,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3779,12 +3767,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -4286,12 +4274,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -4383,12 +4371,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -4480,12 +4468,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -4573,12 +4561,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4666,12 +4654,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4759,12 +4747,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4864,12 +4852,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4961,12 +4949,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -5066,12 +5054,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -5165,12 +5153,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -5254,12 +5242,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -5347,12 +5335,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -5440,12 +5428,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -5533,12 +5521,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -5614,12 +5602,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -5715,12 +5703,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5814,12 +5802,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -5915,12 +5903,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -6018,12 +6006,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -6121,12 +6109,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -6228,12 +6216,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -6327,12 +6315,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -6424,12 +6412,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -6517,12 +6505,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -8700,12 +8688,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -8797,12 +8785,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -8894,12 +8882,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -8991,12 +8979,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -9088,12 +9076,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -9185,12 +9173,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -9237,20 +9225,20 @@
         <v>293</v>
       </c>
       <c r="T90" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="U90" t="n">
         <v>42</v>
       </c>
       <c r="V90" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W90" t="inlineStr"/>
       <c r="X90" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="Y90" t="n">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="Z90" t="inlineStr">
         <is>
@@ -9288,12 +9276,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -9348,10 +9336,10 @@
       <c r="V91" t="inlineStr"/>
       <c r="W91" t="inlineStr"/>
       <c r="X91" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="Y91" t="n">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="Z91" t="inlineStr"/>
       <c r="AA91" t="inlineStr"/>
@@ -9385,12 +9373,12 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -9437,22 +9425,20 @@
         <v>293</v>
       </c>
       <c r="T92" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="U92" t="n">
         <v>18</v>
       </c>
       <c r="V92" t="n">
-        <v>7</v>
-      </c>
-      <c r="W92" t="n">
-        <v>1</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="W92" t="inlineStr"/>
       <c r="X92" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Y92" t="n">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="Z92" t="inlineStr">
         <is>
@@ -9490,12 +9476,12 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -9587,12 +9573,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -9684,12 +9670,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -9781,12 +9767,12 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -9878,12 +9864,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -9975,12 +9961,12 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -10076,12 +10062,12 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -10177,12 +10163,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -10278,12 +10264,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -10379,12 +10365,12 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -10437,16 +10423,16 @@
         <v>272</v>
       </c>
       <c r="V102" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="W102" t="n">
         <v>25</v>
       </c>
       <c r="X102" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y102" t="n">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="Z102" t="inlineStr"/>
       <c r="AA102" t="inlineStr"/>
@@ -10480,12 +10466,12 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -10544,7 +10530,7 @@
         <v>25</v>
       </c>
       <c r="X103" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y103" t="n">
         <v>303</v>
@@ -10585,12 +10571,12 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -10678,12 +10664,12 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -10736,7 +10722,7 @@
         <v>210</v>
       </c>
       <c r="V105" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W105" t="n">
         <v>30</v>
@@ -10745,11 +10731,11 @@
         <v>0</v>
       </c>
       <c r="Y105" t="n">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="Z105" t="inlineStr">
         <is>
-          <t>02/48</t>
+          <t>03/73</t>
         </is>
       </c>
       <c r="AA105" t="inlineStr"/>
@@ -10783,12 +10769,12 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -10841,14 +10827,14 @@
         <v>0</v>
       </c>
       <c r="V106" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="W106" t="inlineStr"/>
       <c r="X106" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y106" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="Z106" t="inlineStr"/>
       <c r="AA106" t="inlineStr"/>
@@ -10882,12 +10868,12 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -10981,12 +10967,12 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -11080,12 +11066,12 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -11179,12 +11165,12 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -11278,12 +11264,12 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -11375,12 +11361,12 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -11472,12 +11458,12 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -11567,12 +11553,12 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -11662,12 +11648,12 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -11757,12 +11743,12 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -11856,12 +11842,12 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -11912,16 +11898,14 @@
         <v>350</v>
       </c>
       <c r="V117" t="n">
-        <v>10</v>
-      </c>
-      <c r="W117" t="n">
-        <v>1</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="W117" t="inlineStr"/>
       <c r="X117" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Y117" t="n">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="Z117" t="inlineStr">
         <is>
@@ -11930,8 +11914,8 @@
       </c>
       <c r="AA117" t="inlineStr">
         <is>
-          <t>Loc-51/3-Casting WIP
-Loc-64/3-Casting Compl
+          <t>Loc-54/1-Casting WIP
+Loc-64/4-Casting WIP
 Loc-74/9-Excavation compl</t>
         </is>
       </c>
@@ -11965,12 +11949,12 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -12060,12 +12044,12 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -12116,14 +12100,14 @@
         <v>310</v>
       </c>
       <c r="V119" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W119" t="inlineStr"/>
       <c r="X119" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Y119" t="n">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="Z119" t="inlineStr">
         <is>
@@ -12132,7 +12116,7 @@
       </c>
       <c r="AA119" t="inlineStr">
         <is>
-          <t>51/4-Tower erection WIP(3rd Section compl)</t>
+          <t>51/4-Tower erection WIP(First Section WIP)</t>
         </is>
       </c>
     </row>
@@ -12165,12 +12149,12 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -12260,12 +12244,12 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -12353,12 +12337,12 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -12446,12 +12430,12 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -12539,12 +12523,12 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -12634,12 +12618,12 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -12729,12 +12713,12 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -12824,12 +12808,12 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -12919,12 +12903,12 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -13014,12 +12998,12 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -13109,12 +13093,12 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -13208,12 +13192,12 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -13264,27 +13248,17 @@
         <v>197</v>
       </c>
       <c r="V131" t="n">
-        <v>1</v>
-      </c>
-      <c r="W131" t="n">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="W131" t="inlineStr"/>
       <c r="X131" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Y131" t="n">
-        <v>196</v>
-      </c>
-      <c r="Z131" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AA131" t="inlineStr">
-        <is>
-          <t>Loc-28/1-Casting  U/P</t>
-        </is>
-      </c>
+        <v>195</v>
+      </c>
+      <c r="Z131" t="inlineStr"/>
+      <c r="AA131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -13315,12 +13289,12 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -13412,12 +13386,12 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -13507,12 +13481,12 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -13600,12 +13574,12 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -13691,12 +13665,12 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -13780,12 +13754,12 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -13869,12 +13843,12 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -13960,12 +13934,12 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -14014,20 +13988,20 @@
         <v>40</v>
       </c>
       <c r="V139" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="W139" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X139" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="Y139" t="n">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="Z139" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="AA139" t="inlineStr"/>
@@ -14061,12 +14035,12 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -14115,16 +14089,16 @@
         <v>40</v>
       </c>
       <c r="V140" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="W140" t="n">
         <v>0</v>
       </c>
       <c r="X140" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="Y140" t="n">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="Z140" t="inlineStr"/>
       <c r="AA140" t="inlineStr"/>
@@ -14158,12 +14132,12 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -14259,12 +14233,12 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -14356,12 +14330,12 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -14453,12 +14427,12 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -14550,12 +14524,12 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -14637,12 +14611,12 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -14724,12 +14698,12 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -14811,12 +14785,12 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -14898,12 +14872,12 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -16030,12 +16004,12 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -16135,12 +16109,12 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -16236,12 +16210,12 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -16341,12 +16315,12 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -16442,12 +16416,12 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -16502,9 +16476,7 @@
       <c r="V165" t="n">
         <v>3</v>
       </c>
-      <c r="W165" t="n">
-        <v>1</v>
-      </c>
+      <c r="W165" t="inlineStr"/>
       <c r="X165" t="n">
         <v>198</v>
       </c>
@@ -16516,11 +16488,7 @@
           <t>0.0</t>
         </is>
       </c>
-      <c r="AA165" t="inlineStr">
-        <is>
-          <t>34/0 erection completed</t>
-        </is>
-      </c>
+      <c r="AA165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -16551,12 +16519,12 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -16656,12 +16624,12 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -16743,12 +16711,12 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -16848,12 +16816,12 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -16949,12 +16917,12 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -17007,16 +16975,16 @@
         <v>10.278165</v>
       </c>
       <c r="V170" t="n">
-        <v>8.527380999999984</v>
+        <v>10.38895099999999</v>
       </c>
       <c r="W170" t="n">
         <v>0</v>
       </c>
       <c r="X170" t="n">
-        <v>62.24921599999998</v>
+        <v>64.11078599999999</v>
       </c>
       <c r="Y170" t="n">
-        <v>1.750784000000017</v>
+        <v>-0.1107859999999903</v>
       </c>
       <c r="Z170" t="inlineStr">
         <is>
@@ -17054,12 +17022,12 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -17153,12 +17121,12 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -17252,12 +17220,12 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -17361,12 +17329,12 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -17466,12 +17434,12 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -17571,12 +17539,12 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -17676,12 +17644,12 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -17761,12 +17729,12 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -17866,12 +17834,12 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -17967,12 +17935,12 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -20696,12 +20664,12 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -20795,12 +20763,12 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -20849,20 +20817,20 @@
         <v>72</v>
       </c>
       <c r="V208" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="W208" t="n">
         <v>2</v>
       </c>
       <c r="X208" t="n">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="Y208" t="n">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="Z208" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>31</t>
         </is>
       </c>
       <c r="AA208" t="inlineStr"/>
@@ -20896,12 +20864,12 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -20950,16 +20918,16 @@
         <v>70</v>
       </c>
       <c r="V209" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="W209" t="n">
         <v>0</v>
       </c>
       <c r="X209" t="n">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="Y209" t="n">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="Z209" t="inlineStr">
         <is>
@@ -20997,12 +20965,12 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
@@ -21051,20 +21019,20 @@
         <v>75</v>
       </c>
       <c r="V210" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="W210" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X210" t="n">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="Y210" t="n">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="Z210" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="AA210" t="inlineStr"/>
@@ -21098,12 +21066,12 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
@@ -21199,12 +21167,12 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
@@ -25122,7 +25090,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -25178,7 +25146,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -25201,7 +25169,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -25255,7 +25223,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -25274,7 +25242,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -25323,12 +25291,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -25418,7 +25386,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -25453,7 +25421,7 @@
       <c r="I6" t="inlineStr">
         <is>
           <t>C3:Activity-&gt;activity_raw; C4:Quantity-&gt;quantity_loa; C5:unnamed_col_5-&gt;quantity_estimated_or_total; C7:unnamed_col_7-&gt;cumulative_last_month; C9:unnamed_col_9-&gt;plan_for_month; C10:Progress for the Month-&gt;progress_for_month; C11:unnamed_col_11-&gt;today_progress; C12:Cumulative Progress-&gt;cumulative_progress; C13:Balance Progress-&gt;balance_progress; C14:Gangs working 
-May-26-&gt;gangs_working; C15:2026-05-21 00:00:00 Remarks-&gt;remarks</t>
+May-26-&gt;gangs_working; C15:2026-05-22 00:00:00 Remarks-&gt;remarks</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -25472,7 +25440,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -25491,7 +25459,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -25540,12 +25508,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -25847,7 +25815,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -25882,7 +25850,7 @@
       <c r="I12" t="inlineStr">
         <is>
           <t>C2:Activity-&gt;activity_raw; C3:Estimated Quantity-&gt;quantity_estimated_or_total; C4:Cumm. Progress up to
-till last Month (Mar'26)-&gt;cumulative_last_month; C6:L3 Plan for the month (April'26 )-&gt;plan_for_month; C7:Today's Progress-&gt;today_progress; C8:Progress in this month-&gt;progress_for_month; C9:Cumm. Progress till date-&gt;cumulative_progress; C10:Cumm. Balance-&gt;balance_progress; C12:No of Gangs-&gt;gangs_working; C13:Remark-&gt;remarks</t>
+till last Month April'26)-&gt;cumulative_last_month; C6:L3 Plan for the month (April'26 )-&gt;plan_for_month; C7:Today's Progress-&gt;today_progress; C8:Progress in this month-&gt;progress_for_month; C9:Cumm. Progress till date-&gt;cumulative_progress; C10:Cumm. Balance-&gt;balance_progress; C12:No of Gangs-&gt;gangs_working; C13:Remark-&gt;remarks</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -25897,7 +25865,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="O12" t="inlineStr"/>
@@ -25916,7 +25884,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -25965,7 +25933,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="O13" t="inlineStr"/>
@@ -25984,7 +25952,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -26036,7 +26004,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="O14" t="inlineStr"/>
@@ -26055,7 +26023,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -26105,12 +26073,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -26200,7 +26168,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -26249,17 +26217,17 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>MATCH</t>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -26418,7 +26386,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -26469,12 +26437,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -26786,7 +26754,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -26804,7 +26772,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -26847,7 +26815,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -26865,7 +26833,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
@@ -26876,7 +26844,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Project Details; 765KV TA 414 VNTL; VNTL - KEC; Sheet5; Sheet3; Sheet1; DPR Sheet; FDN; FDN Completed; Erection ; Erection Completed ; Erection Compiled; Stringing; Stringing Completed; Stringing Compiled; Sheet6; Sheet4; Sheet7; Visual chart; Pile Fdn; Crossing; Sheet2; Survey; Soil Inv.; Survey Anx</t>
+          <t>Project Details; 765KV TA 414 VNTL; VNTL - KEC; DPR Sheet; Sheet5; Sheet3; Sheet1; FDN; FDN Completed; Erection ; Erection Completed ; Erection Compiled; Stringing; Stringing Completed; Stringing Compiled; Sheet6; Sheet4; Sheet7; Visual chart; Pile Fdn; Crossing; Sheet2; Survey; Soil Inv.; Survey Anx</t>
         </is>
       </c>
     </row>
@@ -26904,7 +26872,7 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -26922,12 +26890,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -27026,7 +26994,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -27044,7 +27012,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="K6" t="inlineStr"/>
@@ -27083,7 +27051,7 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -27101,12 +27069,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -27376,7 +27344,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -27394,7 +27362,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
@@ -27433,7 +27401,7 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -27451,7 +27419,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
@@ -27462,7 +27430,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Summary S; Supply Status; Summary E; DPR Sheet ; DS; CS; Hindrance Record; Earthing; Foundation; Erection Compiled; Tack Welding; Visual Chart; WIP; Statuary clearance; Stringing; OPGW; Accessories; Shield Wire Earthing; TS Gantry - AP47; Project Details; Sheet1; L3 Plan; Supply DPR ; Power line Crossings ; Hardware</t>
+          <t>Summary S; Supply Status; Summary E; DPR Sheet ; DS; CS; Hindrance Record; Earthing; Foundation; Erection Compiled; Tack Welding; Visual Chart; WIP; Statuary clearance; Stringing; OPGW; Accessories; Shield Wire Earthing; TS Gantry - AP47; Project Details; L3 Plan; Supply DPR ; Power line Crossings ; Hardware</t>
         </is>
       </c>
     </row>
@@ -27490,7 +27458,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -27508,7 +27476,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
@@ -27608,7 +27576,7 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -27626,12 +27594,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -27779,7 +27747,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-22.xlsx</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -27797,17 +27765,17 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>MATCH</t>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -27954,7 +27922,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -27972,12 +27940,12 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-25 12:16:56
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -4274,12 +4274,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -4371,12 +4371,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -4468,12 +4468,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -4561,12 +4561,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4654,12 +4654,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4747,12 +4747,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4819,7 +4819,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>37/0, 38/2, 39/0, 47/0, 52/1, 52/2, 54/0,  59/0, 65/2, 66/0, 68/0, 70/0,72/0, 73/0, 75/0, 76/0, 76/1, 82/0, 87/1, 95A/0, 96/0</t>
+          <t>37/0, 38/2, 38/4, 39/0, 47/0, 52/1, 52/2, 54/0,  59/0, 65/2, 66/0, 68/0, 70/0,72/0, 73/0, 75/0, 76/0, 76/1, 82/0, 87/1, 95A/0, 96/0, 96/2</t>
         </is>
       </c>
     </row>
@@ -4852,12 +4852,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4949,12 +4949,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -5005,14 +5005,14 @@
         <v>40</v>
       </c>
       <c r="V46" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W46" t="inlineStr"/>
       <c r="X46" t="n">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="Y46" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Z46" t="inlineStr">
         <is>
@@ -5021,7 +5021,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>13/0, 15/0, 14/1, 32/0, 42/0 , 61/0,  62/0,  64/2, 64/3, 81/0</t>
+          <t>13/0, 15/0, 14/1, 32/0, 42/0 , 61/0,  62/0,  64A/0, 64/3, 81/0</t>
         </is>
       </c>
     </row>
@@ -5054,12 +5054,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -5153,12 +5153,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -5242,12 +5242,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -5335,12 +5335,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -5428,12 +5428,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -5521,12 +5521,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -18044,12 +18044,12 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -18147,12 +18147,12 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -18250,12 +18250,12 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -18353,12 +18353,12 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -18456,12 +18456,12 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -18523,12 +18523,12 @@
       </c>
       <c r="Z185" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="AA185" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>54.0</t>
         </is>
       </c>
     </row>
@@ -18565,12 +18565,12 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -18666,12 +18666,12 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -18722,14 +18722,16 @@
         <v>30</v>
       </c>
       <c r="V187" t="n">
-        <v>16</v>
-      </c>
-      <c r="W187" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="W187" t="n">
+        <v>3</v>
+      </c>
       <c r="X187" t="n">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="Y187" t="n">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="Z187" t="inlineStr">
         <is>
@@ -18738,7 +18740,7 @@
       </c>
       <c r="AA187" t="inlineStr">
         <is>
-          <t>141.0</t>
+          <t>120.0</t>
         </is>
       </c>
     </row>
@@ -18775,12 +18777,12 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -18882,12 +18884,12 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -18967,12 +18969,12 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -19025,9 +19027,7 @@
       <c r="V190" t="n">
         <v>3.712</v>
       </c>
-      <c r="W190" t="n">
-        <v>0.165</v>
-      </c>
+      <c r="W190" t="inlineStr"/>
       <c r="X190" t="n">
         <v>21.195</v>
       </c>
@@ -19078,12 +19078,12 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -19134,14 +19134,14 @@
         <v>15.147</v>
       </c>
       <c r="V191" t="n">
-        <v>3.486</v>
+        <v>3.651</v>
       </c>
       <c r="W191" t="inlineStr"/>
       <c r="X191" t="n">
-        <v>20.532</v>
+        <v>20.697</v>
       </c>
       <c r="Y191" t="n">
-        <v>168.146</v>
+        <v>167.981</v>
       </c>
       <c r="Z191" t="inlineStr"/>
       <c r="AA191" t="inlineStr"/>
@@ -19179,12 +19179,12 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -19272,12 +19272,12 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -19367,12 +19367,12 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -19462,12 +19462,12 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -19565,12 +19565,12 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -19668,12 +19668,12 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -19771,12 +19771,12 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -19874,12 +19874,12 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -19930,25 +19930,25 @@
         <v>11</v>
       </c>
       <c r="V199" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="W199" t="n">
         <v>1</v>
       </c>
       <c r="X199" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="Y199" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Z199" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="AA199" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>35.0</t>
         </is>
       </c>
     </row>
@@ -19985,12 +19985,12 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -20088,12 +20088,12 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -20195,12 +20195,12 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -20290,12 +20290,12 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -20377,12 +20377,12 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -20474,12 +20474,12 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -20571,12 +20571,12 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -25386,7 +25386,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -25421,7 +25421,7 @@
       <c r="I6" t="inlineStr">
         <is>
           <t>C3:Activity-&gt;activity_raw; C4:Quantity-&gt;quantity_loa; C5:unnamed_col_5-&gt;quantity_estimated_or_total; C7:unnamed_col_7-&gt;cumulative_last_month; C9:unnamed_col_9-&gt;plan_for_month; C10:Progress for the Month-&gt;progress_for_month; C11:unnamed_col_11-&gt;today_progress; C12:Cumulative Progress-&gt;cumulative_progress; C13:Balance Progress-&gt;balance_progress; C14:Gangs working 
-May-26-&gt;gangs_working; C15:2026-05-22 00:00:00 Remarks-&gt;remarks</t>
+May-26-&gt;gangs_working; C15:2026-05-24 00:00:00 Remarks-&gt;remarks</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -25440,7 +25440,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -26240,7 +26240,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -26294,7 +26294,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="O18" t="inlineStr"/>
@@ -26313,7 +26313,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -26367,7 +26367,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="O19" t="inlineStr"/>
@@ -26994,7 +26994,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -27012,7 +27012,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="K6" t="inlineStr"/>
@@ -27808,7 +27808,7 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -27826,7 +27826,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
@@ -27865,7 +27865,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-21.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -27883,7 +27883,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-25 16:14:53
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -6598,12 +6598,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -6640,10 +6640,10 @@
       </c>
       <c r="Q63" t="inlineStr"/>
       <c r="R63" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="S63" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="T63" t="n">
         <v>69</v>
@@ -6655,7 +6655,7 @@
         <v>69</v>
       </c>
       <c r="Y63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z63" t="inlineStr"/>
       <c r="AA63" t="inlineStr"/>
@@ -6689,12 +6689,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -6731,10 +6731,10 @@
       </c>
       <c r="Q64" t="inlineStr"/>
       <c r="R64" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="S64" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="T64" t="n">
         <v>67</v>
@@ -6748,7 +6748,7 @@
         <v>67</v>
       </c>
       <c r="Y64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Z64" t="inlineStr"/>
       <c r="AA64" t="inlineStr"/>
@@ -6782,12 +6782,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -6824,10 +6824,10 @@
       </c>
       <c r="Q65" t="inlineStr"/>
       <c r="R65" t="n">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="S65" t="n">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="T65" t="n">
         <v>139</v>
@@ -6836,14 +6836,14 @@
         <v>29</v>
       </c>
       <c r="V65" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W65" t="inlineStr"/>
       <c r="X65" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="Y65" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="Z65" t="inlineStr"/>
       <c r="AA65" t="inlineStr"/>
@@ -6877,12 +6877,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -6919,10 +6919,10 @@
       </c>
       <c r="Q66" t="inlineStr"/>
       <c r="R66" t="n">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="S66" t="n">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="T66" t="n">
         <v>121</v>
@@ -6936,7 +6936,7 @@
         <v>121</v>
       </c>
       <c r="Y66" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="Z66" t="inlineStr"/>
       <c r="AA66" t="inlineStr"/>
@@ -6970,12 +6970,12 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -7063,12 +7063,12 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -7105,10 +7105,10 @@
       </c>
       <c r="Q68" t="inlineStr"/>
       <c r="R68" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="S68" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="T68" t="inlineStr"/>
       <c r="U68" t="inlineStr"/>
@@ -7118,7 +7118,7 @@
         <v>0</v>
       </c>
       <c r="Y68" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="Z68" t="inlineStr"/>
       <c r="AA68" t="inlineStr"/>
@@ -7742,12 +7742,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -7833,12 +7833,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -7924,12 +7924,12 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -8019,12 +8019,12 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -8073,11 +8073,11 @@
         <v>46</v>
       </c>
       <c r="V78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="n">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="Y78" t="n">
         <v>202</v>
@@ -8114,12 +8114,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -8168,11 +8168,11 @@
         <v>38</v>
       </c>
       <c r="V79" t="n">
-        <v>10.157</v>
+        <v>10.629</v>
       </c>
       <c r="W79" t="inlineStr"/>
       <c r="X79" t="n">
-        <v>53.72499999999999</v>
+        <v>54.197</v>
       </c>
       <c r="Y79" t="n">
         <v>179.432</v>
@@ -8209,12 +8209,12 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -25531,7 +25531,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -25584,7 +25584,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O8" t="inlineStr"/>
@@ -25671,7 +25671,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -25724,7 +25724,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O10" t="inlineStr"/>
@@ -27112,7 +27112,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -27130,7 +27130,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
@@ -27226,7 +27226,7 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -27244,7 +27244,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="K10" t="inlineStr"/>
@@ -27255,7 +27255,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>DPR_TA-506; Erection compiled; Tightening; Stringing; Visual Chart; Project Details; Location Summary</t>
+          <t>DPR_TA-506; Erection compiled; Tightening; Stringing; VC; Project Details; Location Summary</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-26 16:07:49
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -17646,12 +17646,12 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -17749,12 +17749,12 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -17852,12 +17852,12 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -17955,12 +17955,12 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -18058,12 +18058,12 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -18167,12 +18167,12 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -18268,12 +18268,12 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -18326,9 +18326,7 @@
       <c r="V183" t="n">
         <v>19</v>
       </c>
-      <c r="W183" t="n">
-        <v>3</v>
-      </c>
+      <c r="W183" t="inlineStr"/>
       <c r="X183" t="n">
         <v>213</v>
       </c>
@@ -18379,12 +18377,12 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -18486,12 +18484,12 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -18571,12 +18569,12 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -18627,14 +18625,14 @@
         <v>15.147</v>
       </c>
       <c r="V186" t="n">
-        <v>3.712</v>
+        <v>3.877</v>
       </c>
       <c r="W186" t="inlineStr"/>
       <c r="X186" t="n">
-        <v>21.195</v>
+        <v>21.36</v>
       </c>
       <c r="Y186" t="n">
-        <v>167.483</v>
+        <v>167.318</v>
       </c>
       <c r="Z186" t="inlineStr">
         <is>
@@ -18680,12 +18678,12 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -18736,14 +18734,16 @@
         <v>15.147</v>
       </c>
       <c r="V187" t="n">
-        <v>3.651</v>
-      </c>
-      <c r="W187" t="inlineStr"/>
+        <v>3.877</v>
+      </c>
+      <c r="W187" t="n">
+        <v>0.226</v>
+      </c>
       <c r="X187" t="n">
-        <v>20.697</v>
+        <v>20.923</v>
       </c>
       <c r="Y187" t="n">
-        <v>167.981</v>
+        <v>167.755</v>
       </c>
       <c r="Z187" t="inlineStr"/>
       <c r="AA187" t="inlineStr"/>
@@ -18781,12 +18781,12 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -18874,12 +18874,12 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -18969,12 +18969,12 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -19064,12 +19064,12 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -19167,12 +19167,12 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -19270,12 +19270,12 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -19373,12 +19373,12 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -19476,12 +19476,12 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -19534,9 +19534,7 @@
       <c r="V195" t="n">
         <v>10</v>
       </c>
-      <c r="W195" t="n">
-        <v>1</v>
-      </c>
+      <c r="W195" t="inlineStr"/>
       <c r="X195" t="n">
         <v>32</v>
       </c>
@@ -19587,12 +19585,12 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -19690,12 +19688,12 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -19797,12 +19795,12 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -19892,12 +19890,12 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -19979,12 +19977,12 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -20076,12 +20074,12 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -20173,12 +20171,12 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -25842,7 +25840,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -25896,7 +25894,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O18" t="inlineStr"/>
@@ -25915,7 +25913,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -25969,7 +25967,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="O19" t="inlineStr"/>
@@ -27410,7 +27408,7 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -27428,7 +27426,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
@@ -27439,7 +27437,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>400kV Summery; Check Survey ; Check Survey Status; Check Survey; Sheet8; Sheet2; Project Details; Statutory Clearence;  Crossing Proposal; Sheet1; VC 51-96; VC; ROW; June; Foundation; Royalty; Sheet14; Sheet7; Erection ; Completion date; Erection Compiled ; Earthing; Final Check In And Tack Welding; Sheet10; Stringing Compiled ; Soil Investigation; Sheet9; VC ; Sheet6; VC 51-121; Sheet5; Sheet3; Tower Schedule; Visual Chart; L2 Vs Actual Progress Chart; L2 Vs Actual Progress Chart (2); Sheet4</t>
+          <t>400kV Summery; Check Survey ; Check Survey Status; Check Survey; Sheet8; Sheet2; Project Details; Statutory Clearence;  Crossing Proposal; Sheet1; VC 51-96; VC; ROW; June; Foundation; Royalty; Sheet14; Sheet7; Erection ; Completion date; Erection Compiled ; Earthing; Final Check In And Tack Welding; Sheet10; Stringing Compiled ; Soil Investigation; Sheet9; VC ; Sheet6; VC 51-121; Sheet5; Sheet3; Tower Schedule; Visual Chart 1; Visual Chart; L2 Vs Actual Progress Chart; L2 Vs Actual Progress Chart (2); Sheet4</t>
         </is>
       </c>
     </row>
@@ -27467,7 +27465,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-24.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -27485,7 +27483,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-27 10:45:24
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -1819,12 +1819,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1910,12 +1910,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2001,12 +2001,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2092,12 +2092,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2183,12 +2183,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2278,12 +2278,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2377,12 +2377,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2472,12 +2472,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2526,16 +2526,16 @@
         <v>55</v>
       </c>
       <c r="V21" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="W21" t="n">
         <v>1</v>
       </c>
       <c r="X21" t="n">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="Y21" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
@@ -2577,12 +2577,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2631,14 +2631,16 @@
         <v>55</v>
       </c>
       <c r="V22" t="n">
-        <v>17</v>
-      </c>
-      <c r="W22" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="W22" t="n">
+        <v>2</v>
+      </c>
       <c r="X22" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="Y22" t="n">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -2676,12 +2678,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2730,14 +2732,14 @@
         <v>20</v>
       </c>
       <c r="V23" t="n">
-        <v>6.052</v>
+        <v>7.379</v>
       </c>
       <c r="W23" t="inlineStr"/>
       <c r="X23" t="n">
-        <v>12.68</v>
+        <v>14.007</v>
       </c>
       <c r="Y23" t="n">
-        <v>115.119</v>
+        <v>113.792</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -2775,12 +2777,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2831,7 +2833,9 @@
       <c r="V24" t="n">
         <v>6.401</v>
       </c>
-      <c r="W24" t="inlineStr"/>
+      <c r="W24" t="n">
+        <v>1.327</v>
+      </c>
       <c r="X24" t="n">
         <v>18.097</v>
       </c>
@@ -2870,12 +2874,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2924,14 +2928,16 @@
         <v>20</v>
       </c>
       <c r="V25" t="n">
-        <v>6.052</v>
-      </c>
-      <c r="W25" t="inlineStr"/>
+        <v>7.379</v>
+      </c>
+      <c r="W25" t="n">
+        <v>1.327</v>
+      </c>
       <c r="X25" t="n">
-        <v>12.68</v>
+        <v>14.007</v>
       </c>
       <c r="Y25" t="n">
-        <v>115.119</v>
+        <v>113.792</v>
       </c>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="inlineStr"/>
@@ -2965,12 +2971,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -3058,12 +3064,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -3159,12 +3165,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -3260,12 +3266,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3361,12 +3367,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -5196,12 +5202,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -5297,12 +5303,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -5396,12 +5402,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -5497,12 +5503,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -5555,18 +5561,18 @@
         <v>40</v>
       </c>
       <c r="V52" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="W52" t="inlineStr"/>
       <c r="X52" t="n">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="Y52" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="AA52" t="inlineStr"/>
@@ -5600,12 +5606,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -5703,12 +5709,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5761,23 +5767,25 @@
         <v>14.192</v>
       </c>
       <c r="V54" t="n">
-        <v>6.211</v>
-      </c>
-      <c r="W54" t="inlineStr"/>
+        <v>8.317</v>
+      </c>
+      <c r="W54" t="n">
+        <v>0.248</v>
+      </c>
       <c r="X54" t="n">
-        <v>113.361</v>
+        <v>115.467</v>
       </c>
       <c r="Y54" t="n">
-        <v>7.980999999999995</v>
+        <v>5.874999999999986</v>
       </c>
       <c r="Z54" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>35/0 - 36/0 - Conductor payingout under progreess +34/2 -35/0 - Conductor passing under progress + 33/0 -34/0 - Insualtor Hosting under progress</t>
+          <t>33/0 -34/0 - Top phase payingout under progress  + 34/0- 34/1 - PP rope passing done  + 34/1 -  34/2 - Insulator hosting done</t>
         </is>
       </c>
     </row>
@@ -5810,12 +5818,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -5868,17 +5876,23 @@
         <v>14.192</v>
       </c>
       <c r="V55" t="n">
-        <v>6.21075</v>
-      </c>
-      <c r="W55" t="inlineStr"/>
+        <v>6.45875</v>
+      </c>
+      <c r="W55" t="n">
+        <v>0.248</v>
+      </c>
       <c r="X55" t="n">
-        <v>113.36075</v>
+        <v>113.60875</v>
       </c>
       <c r="Y55" t="n">
-        <v>7.981249999999989</v>
+        <v>7.733249999999998</v>
       </c>
       <c r="Z55" t="inlineStr"/>
-      <c r="AA55" t="inlineStr"/>
+      <c r="AA55" t="inlineStr">
+        <is>
+          <t>Bottom phase final sag planned for tomorrow</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5909,12 +5923,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -6006,12 +6020,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -6099,12 +6113,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -8282,12 +8296,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -8379,12 +8393,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -8476,12 +8490,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -8573,12 +8587,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -8670,12 +8684,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -8767,12 +8781,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -8825,14 +8839,14 @@
         <v>42</v>
       </c>
       <c r="V86" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W86" t="inlineStr"/>
       <c r="X86" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="Y86" t="n">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="Z86" t="inlineStr">
         <is>
@@ -8870,12 +8884,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -8967,12 +8981,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -9070,12 +9084,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -9167,12 +9181,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -9264,12 +9278,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -9361,12 +9375,12 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -9458,12 +9472,12 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -9555,12 +9569,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -9656,12 +9670,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -9757,12 +9771,12 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -9858,12 +9872,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -9959,12 +9973,12 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -10060,12 +10074,12 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -10124,7 +10138,7 @@
         <v>25</v>
       </c>
       <c r="X99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y99" t="n">
         <v>304</v>
@@ -10165,12 +10179,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -10258,12 +10272,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -10316,16 +10330,16 @@
         <v>210</v>
       </c>
       <c r="V101" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W101" t="n">
         <v>30</v>
       </c>
       <c r="X101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y101" t="n">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="Z101" t="inlineStr">
         <is>
@@ -10363,12 +10377,12 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -10462,12 +10476,12 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -10561,12 +10575,12 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -10660,12 +10674,12 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -10759,12 +10773,12 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -10858,12 +10872,12 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -10955,12 +10969,12 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -11052,12 +11066,12 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -11147,12 +11161,12 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -11242,12 +11256,12 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -11337,12 +11351,12 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -11436,12 +11450,12 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -11492,25 +11506,28 @@
         <v>350</v>
       </c>
       <c r="V113" t="n">
-        <v>11</v>
-      </c>
-      <c r="W113" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="W113" t="n">
+        <v>1</v>
+      </c>
       <c r="X113" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Y113" t="n">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="Z113" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AA113" t="inlineStr">
         <is>
           <t>Loc-54/1-Casting WIP
-Loc-64/4-Casting WIP
-Loc-74/9-Excavation compl</t>
+Loc-74/9-Casting WIP
+Loc-64/6-Casting WIP
+Loc-61/2-Steel binding WIP</t>
         </is>
       </c>
     </row>
@@ -11543,12 +11560,12 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -11638,12 +11655,12 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -11710,7 +11727,7 @@
       </c>
       <c r="AA115" t="inlineStr">
         <is>
-          <t>51/4-Tower erection WIP(First Section WIP)</t>
+          <t>51/4-Tower erection WIP(Second Section compl)</t>
         </is>
       </c>
     </row>
@@ -11743,12 +11760,12 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -11838,12 +11855,12 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -11931,12 +11948,12 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -12024,12 +12041,12 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -12117,12 +12134,12 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -12212,12 +12229,12 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -12307,12 +12324,12 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -12402,12 +12419,12 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -12497,12 +12514,12 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -12592,12 +12609,12 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -12687,12 +12704,12 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -12786,12 +12803,12 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -12883,12 +12900,12 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -12980,12 +12997,12 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -13075,12 +13092,12 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -13168,12 +13185,12 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -13259,12 +13276,12 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -13348,12 +13365,12 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -13437,12 +13454,12 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -13528,12 +13545,12 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -13629,12 +13646,12 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -13726,12 +13743,12 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -13827,12 +13844,12 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -13924,12 +13941,12 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -14021,12 +14038,12 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -14118,12 +14135,12 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -14205,12 +14222,12 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -14292,12 +14309,12 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -14379,12 +14396,12 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -14466,12 +14483,12 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -20264,12 +20281,12 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -20363,12 +20380,12 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -20417,16 +20434,16 @@
         <v>72</v>
       </c>
       <c r="V204" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="W204" t="n">
         <v>3</v>
       </c>
       <c r="X204" t="n">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="Y204" t="n">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="Z204" t="inlineStr">
         <is>
@@ -20464,12 +20481,12 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -20518,16 +20535,16 @@
         <v>70</v>
       </c>
       <c r="V205" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="W205" t="n">
         <v>0</v>
       </c>
       <c r="X205" t="n">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="Y205" t="n">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="Z205" t="inlineStr">
         <is>
@@ -20565,12 +20582,12 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -20619,16 +20636,16 @@
         <v>75</v>
       </c>
       <c r="V206" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="W206" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X206" t="n">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="Y206" t="n">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="Z206" t="inlineStr">
         <is>
@@ -20666,12 +20683,12 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -20767,12 +20784,12 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -24769,7 +24786,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -24823,7 +24840,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -24842,7 +24859,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -24891,12 +24908,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -25059,7 +25076,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -25108,12 +25125,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -25415,7 +25432,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -25465,7 +25482,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O12" t="inlineStr"/>
@@ -25484,7 +25501,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -25533,7 +25550,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O13" t="inlineStr"/>
@@ -25552,7 +25569,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -25604,7 +25621,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O14" t="inlineStr"/>
@@ -25623,7 +25640,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -25673,12 +25690,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -25986,7 +26003,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -26037,12 +26054,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -26415,7 +26432,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -26433,7 +26450,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
@@ -26472,7 +26489,7 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -26490,12 +26507,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -26651,7 +26668,7 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-22.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -26669,12 +26686,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -26944,7 +26961,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -26962,7 +26979,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
@@ -27001,7 +27018,7 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -27019,7 +27036,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
@@ -27058,7 +27075,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>TA 513 - DPR - 2026-05-24.xlsx</t>
+          <t>TA 513 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -27076,7 +27093,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
@@ -27176,7 +27193,7 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -27194,12 +27211,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -27522,7 +27539,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -27540,12 +27557,12 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-27 11:46:57
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -3874,12 +3874,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3971,12 +3971,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -4068,12 +4068,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -4161,12 +4161,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -4254,12 +4254,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -4347,12 +4347,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -4403,14 +4403,14 @@
         <v>45</v>
       </c>
       <c r="V40" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="n">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="Y40" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="Z40" t="inlineStr">
         <is>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="AA40" t="inlineStr">
         <is>
-          <t>37/0, 38/2, 38/4, 39/0, 47/0, 52/1, 52/2, 59/0, 65/2, 66/0, 68/0, 70/0,72/0, 73/0, 75/0, 76/0, 76/1, 82/0, 87/1, 95A/0, 96/0, 96/2</t>
+          <t>38/2, 38/4, 39/0, 47/0, 52/1, 52/2, 59/0, 65/2, 66/0, 68/0, 70/0,72/0, 73/0, 75/0, 76/0, 76/1, 82/0, 87/1, 95A/0, 96/0, 96/2</t>
         </is>
       </c>
     </row>
@@ -4452,12 +4452,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -4549,12 +4549,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4605,14 +4605,14 @@
         <v>40</v>
       </c>
       <c r="V42" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="W42" t="inlineStr"/>
       <c r="X42" t="n">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="Y42" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="Z42" t="inlineStr">
         <is>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="AA42" t="inlineStr">
         <is>
-          <t>13/0, 15/0, 14/1, 32/0, 42/0 , 61/0,  62/0,  64A/0, 64/3, 81/0</t>
+          <t>13/0, 15/0, 14/1, 32/0, 42/0 ,53/0  62/0,  64A/0, 64/3, 81/0</t>
         </is>
       </c>
     </row>
@@ -4654,12 +4654,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4753,12 +4753,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4842,12 +4842,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4935,12 +4935,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -5028,12 +5028,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -5121,12 +5121,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -25003,7 +25003,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -25038,7 +25038,7 @@
       <c r="I6" t="inlineStr">
         <is>
           <t>C3:Activity-&gt;activity_raw; C4:Quantity-&gt;quantity_loa; C5:unnamed_col_5-&gt;quantity_estimated_or_total; C7:unnamed_col_7-&gt;cumulative_last_month; C9:unnamed_col_9-&gt;plan_for_month; C10:Progress for the Month-&gt;progress_for_month; C11:unnamed_col_11-&gt;today_progress; C12:Cumulative Progress-&gt;cumulative_progress; C13:Balance Progress-&gt;balance_progress; C14:Gangs working 
-May-26-&gt;gangs_working; C15:2026-05-25 00:00:00 Remarks-&gt;remarks</t>
+May-26-&gt;gangs_working; C15:2026-05-26 00:00:00 Remarks-&gt;remarks</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -25057,7 +25057,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -26611,7 +26611,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -26629,7 +26629,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="K6" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-27 12:20:04
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -6206,12 +6206,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -6297,12 +6297,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -6390,12 +6390,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -6485,12 +6485,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -6578,12 +6578,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -6671,12 +6671,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -7350,12 +7350,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -7441,12 +7441,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -7532,12 +7532,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -7586,11 +7586,11 @@
         <v>40</v>
       </c>
       <c r="V73" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W73" t="inlineStr"/>
       <c r="X73" t="n">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="Y73" t="n">
         <v>123</v>
@@ -7627,12 +7627,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -7722,12 +7722,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -7817,12 +7817,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -25148,7 +25148,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -25201,7 +25201,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O8" t="inlineStr"/>
@@ -25288,7 +25288,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -25341,7 +25341,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O10" t="inlineStr"/>
@@ -26729,7 +26729,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -26747,7 +26747,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
@@ -26843,7 +26843,7 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -26861,7 +26861,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="K10" t="inlineStr"/>
@@ -26872,7 +26872,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>DPR_TA-506; Erection compiled; Tightening; Stringing; VC; Project Details; Location Summary</t>
+          <t>DPR_TA-506; VC; Erection compiled; Tightening; Stringing; Project Details; Location Summary</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-28 10:47:26
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -597,12 +597,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -698,12 +698,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -799,12 +799,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -900,12 +900,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1003,12 +1003,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1106,12 +1106,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1205,12 +1205,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1363,7 +1363,7 @@
         <v>31</v>
       </c>
       <c r="W9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X9" t="n">
         <v>255</v>
@@ -1411,12 +1411,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1467,16 +1467,16 @@
         <v>18</v>
       </c>
       <c r="V10" t="n">
-        <v>6.052</v>
+        <v>8.6</v>
       </c>
       <c r="W10" t="n">
-        <v>0</v>
+        <v>2.548</v>
       </c>
       <c r="X10" t="n">
-        <v>74.64099999999999</v>
+        <v>77.18899999999999</v>
       </c>
       <c r="Y10" t="n">
-        <v>43.209851</v>
+        <v>40.661851</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
@@ -1518,12 +1518,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1621,12 +1621,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1677,16 +1677,16 @@
         <v>18</v>
       </c>
       <c r="V12" t="n">
-        <v>6.052</v>
+        <v>8.6</v>
       </c>
       <c r="W12" t="n">
-        <v>0</v>
+        <v>2.548</v>
       </c>
       <c r="X12" t="n">
-        <v>74.64099999999999</v>
+        <v>77.18899999999999</v>
       </c>
       <c r="Y12" t="n">
-        <v>43.209851</v>
+        <v>40.661851</v>
       </c>
       <c r="Z12" t="inlineStr"/>
       <c r="AA12" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1819,12 +1819,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1910,12 +1910,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2001,12 +2001,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2092,12 +2092,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2183,12 +2183,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2278,12 +2278,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2377,12 +2377,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2472,12 +2472,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2526,16 +2526,16 @@
         <v>55</v>
       </c>
       <c r="V21" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="W21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X21" t="n">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="Y21" t="n">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
@@ -2544,7 +2544,7 @@
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>1 gang arrived on 18.05.26</t>
+          <t>1 gang arrived on 27.05.26</t>
         </is>
       </c>
     </row>
@@ -2577,12 +2577,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2631,16 +2631,16 @@
         <v>55</v>
       </c>
       <c r="V22" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="W22" t="n">
         <v>2</v>
       </c>
       <c r="X22" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="Y22" t="n">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -2678,12 +2678,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2777,12 +2777,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2874,12 +2874,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2971,12 +2971,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -3064,12 +3064,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -3165,12 +3165,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -3266,12 +3266,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3367,12 +3367,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -3421,16 +3421,16 @@
         <v>8.4</v>
       </c>
       <c r="V30" t="n">
-        <v>4.051</v>
+        <v>4.41</v>
       </c>
       <c r="W30" t="n">
-        <v>0</v>
+        <v>0.359</v>
       </c>
       <c r="X30" t="n">
-        <v>110.774</v>
+        <v>111.133</v>
       </c>
       <c r="Y30" t="n">
-        <v>4.359999999999985</v>
+        <v>4.000999999999991</v>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
@@ -5202,12 +5202,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -5303,12 +5303,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -5402,12 +5402,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -5503,12 +5503,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -5606,12 +5606,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -5709,12 +5709,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5769,9 +5769,7 @@
       <c r="V54" t="n">
         <v>8.317</v>
       </c>
-      <c r="W54" t="n">
-        <v>0.248</v>
-      </c>
+      <c r="W54" t="inlineStr"/>
       <c r="X54" t="n">
         <v>115.467</v>
       </c>
@@ -5818,12 +5816,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -5878,9 +5876,7 @@
       <c r="V55" t="n">
         <v>6.45875</v>
       </c>
-      <c r="W55" t="n">
-        <v>0.248</v>
-      </c>
+      <c r="W55" t="inlineStr"/>
       <c r="X55" t="n">
         <v>113.60875</v>
       </c>
@@ -5888,11 +5884,7 @@
         <v>7.733249999999998</v>
       </c>
       <c r="Z55" t="inlineStr"/>
-      <c r="AA55" t="inlineStr">
-        <is>
-          <t>Bottom phase final sag planned for tomorrow</t>
-        </is>
-      </c>
+      <c r="AA55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5923,12 +5915,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -6020,12 +6012,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -6113,12 +6105,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -8296,12 +8288,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -8393,12 +8385,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -8490,12 +8482,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -8587,12 +8579,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -8684,12 +8676,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -8781,12 +8773,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -8839,18 +8831,18 @@
         <v>42</v>
       </c>
       <c r="V86" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="W86" t="inlineStr"/>
       <c r="X86" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Y86" t="n">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="Z86" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="AA86" t="inlineStr"/>
@@ -8884,12 +8876,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -8981,12 +8973,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -9084,12 +9076,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -9181,12 +9173,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -9278,12 +9270,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -9375,12 +9367,12 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -9472,12 +9464,12 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -9569,12 +9561,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -9670,12 +9662,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -9771,12 +9763,12 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -9872,12 +9864,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -9973,12 +9965,12 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -10074,12 +10066,12 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -10179,12 +10171,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -10272,12 +10264,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -10330,7 +10322,7 @@
         <v>210</v>
       </c>
       <c r="V101" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W101" t="n">
         <v>30</v>
@@ -10339,7 +10331,7 @@
         <v>1</v>
       </c>
       <c r="Y101" t="n">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="Z101" t="inlineStr">
         <is>
@@ -10377,12 +10369,12 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -10476,12 +10468,12 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -10575,12 +10567,12 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -10674,12 +10666,12 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -10773,12 +10765,12 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -13545,12 +13537,12 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -13646,12 +13638,12 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -13743,12 +13735,12 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -13844,12 +13836,12 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -13941,12 +13933,12 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -14038,12 +14030,12 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -14135,12 +14127,12 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -14222,12 +14214,12 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -14309,12 +14301,12 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -14396,12 +14388,12 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -14483,12 +14475,12 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -14564,12 +14556,12 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -14663,12 +14655,12 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -14760,12 +14752,12 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -14845,12 +14837,12 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -14930,12 +14922,12 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -14990,20 +14982,20 @@
         <v>35</v>
       </c>
       <c r="V150" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="W150" t="n">
         <v>1</v>
       </c>
       <c r="X150" t="n">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="Y150" t="n">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="Z150" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="AA150" t="inlineStr"/>
@@ -15037,12 +15029,12 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -15138,12 +15130,12 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -15227,12 +15219,12 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -15316,12 +15308,12 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -15411,12 +15403,12 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -15508,12 +15500,12 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -15568,16 +15560,16 @@
         <v>40</v>
       </c>
       <c r="V156" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="W156" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X156" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="Y156" t="n">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="Z156" t="inlineStr">
         <is>
@@ -15615,12 +15607,12 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -15720,12 +15712,12 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -15821,12 +15813,12 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -15926,12 +15918,12 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -16027,12 +16019,12 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -16134,12 +16126,12 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -16239,12 +16231,12 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -16295,7 +16287,11 @@
       <c r="X163" t="inlineStr"/>
       <c r="Y163" t="inlineStr"/>
       <c r="Z163" t="inlineStr"/>
-      <c r="AA163" t="inlineStr"/>
+      <c r="AA163" t="inlineStr">
+        <is>
+          <t>33/1 to 33/0 all phase conductor paying out done.</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -16326,12 +16322,12 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -16384,16 +16380,16 @@
         <v>2.799999999999997</v>
       </c>
       <c r="V164" t="n">
-        <v>-0.0007370000000079813</v>
+        <v>1.651832999999989</v>
       </c>
       <c r="W164" t="n">
         <v>0</v>
       </c>
       <c r="X164" t="n">
-        <v>61.19926299999999</v>
+        <v>62.85183299999999</v>
       </c>
       <c r="Y164" t="n">
-        <v>2.800737000000005</v>
+        <v>1.148167000000008</v>
       </c>
       <c r="Z164" t="inlineStr">
         <is>
@@ -16431,12 +16427,12 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -16532,12 +16528,12 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -16637,12 +16633,12 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -16736,12 +16732,12 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -16835,12 +16831,12 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -16944,12 +16940,12 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -17049,12 +17045,12 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -17154,12 +17150,12 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -17259,12 +17255,12 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -17344,12 +17340,12 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -17453,12 +17449,12 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -17554,12 +17550,12 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -20281,12 +20277,12 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-26.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -20380,12 +20376,12 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-26.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -20437,7 +20433,7 @@
         <v>51</v>
       </c>
       <c r="W204" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X204" t="n">
         <v>357</v>
@@ -20481,12 +20477,12 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-26.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -20582,12 +20578,12 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-26.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -20636,16 +20632,16 @@
         <v>75</v>
       </c>
       <c r="V206" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="W206" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X206" t="n">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="Y206" t="n">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="Z206" t="inlineStr">
         <is>
@@ -20683,12 +20679,12 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-26.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -20784,12 +20780,12 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-26.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -24707,7 +24703,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -24763,7 +24759,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -24786,7 +24782,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -24840,7 +24836,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -24859,7 +24855,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -24908,12 +24904,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -25076,7 +25072,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -25125,12 +25121,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -25432,7 +25428,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -25482,7 +25478,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O12" t="inlineStr"/>
@@ -25501,7 +25497,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -25550,7 +25546,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O13" t="inlineStr"/>
@@ -25640,7 +25636,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -25690,12 +25686,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -25713,7 +25709,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -25762,12 +25758,12 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -25785,7 +25781,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -25834,12 +25830,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -26003,7 +25999,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-26.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -26054,12 +26050,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -26371,7 +26367,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-25.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -26389,7 +26385,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -26404,7 +26400,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>TA413_PBNTL; Visual Chart; Stretch readiness ; Stringing; Erection; L2 Plan vs Actual; Survey summary; Detailed Survey ; Check Survey ; Earthing; Tack Welding;  Final checking; Bird Guard ; Accessories; OPGW; Foundation; JUMPER Details; ROW Tracker; S-Curve FDN; S-Curve Erection; S-Curve Stringing; Supply Status; Hardware Supply; Crossing status; Tower Abstract sheet; Statutory Proposals; Tower Abstarct ; Location Summary; Foundation Daily Progress; Tower PRS abstract ; Stretch readiness  (2); Area</t>
+          <t>TA413_PBNTL; Visual Chart; Stringing; Stretch readiness ; Erection; L2 Plan vs Actual; Survey summary; Detailed Survey ; Check Survey ; Earthing; Tack Welding;  Final checking; Bird Guard ; Accessories; OPGW; Foundation; JUMPER Details; ROW Tracker; S-Curve FDN; S-Curve Erection; S-Curve Stringing; Supply Status; Hardware Supply; Crossing status; Tower Abstract sheet; Statutory Proposals; Tower Abstarct ; Location Summary; Foundation Daily Progress; Tower PRS abstract ; Stretch readiness  (2); Area</t>
         </is>
       </c>
     </row>
@@ -26432,7 +26428,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -26450,7 +26446,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
@@ -26489,7 +26485,7 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -26507,12 +26503,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -26668,7 +26664,7 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -26686,12 +26682,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -26961,7 +26957,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -26979,7 +26975,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
@@ -27018,7 +27014,7 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -27036,7 +27032,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
@@ -27193,7 +27189,7 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -27211,12 +27207,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -27226,7 +27222,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Visual Chart ; Master Sheet; Progress Sheet ; ROW; SUPPLY; Erection Compiled; X-ing Details ; Visual Chart; Foundation &amp; Erection; STRG Stretch ; Stringing Compiled</t>
+          <t>Visual Chart ; Master Sheet; Progress Sheet ; SUPPLY; Erection Compiled; X-ing Details ; Visual Chart; Foundation &amp; Erection; STRG Stretch ; Stringing Compiled</t>
         </is>
       </c>
     </row>
@@ -27254,7 +27250,7 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -27272,12 +27268,12 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -27287,7 +27283,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>DPR-KEC; Survey details; FDN; Erection; Visual Chart ; Detail Survey; Check Survey ; Composite-Survey(05-04-2026); Earthing; WIP; statuary clearance; statuary clearance (2); Supply Status</t>
+          <t>DPR-KEC; Survey details; FDN; Erection; WIP; Visual Chart ; Detail Survey; Check Survey ; Composite-Survey(05-04-2026); Earthing; statuary clearance; Supply Status</t>
         </is>
       </c>
     </row>
@@ -27364,7 +27360,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -27382,12 +27378,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -27539,7 +27535,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-26.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -27557,12 +27553,12 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-28 11:51:32
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -3874,12 +3874,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3971,12 +3971,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -4068,12 +4068,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -4161,12 +4161,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -4254,12 +4254,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -4347,12 +4347,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -4452,12 +4452,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -4549,12 +4549,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4605,14 +4605,14 @@
         <v>40</v>
       </c>
       <c r="V42" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="W42" t="inlineStr"/>
       <c r="X42" t="n">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="Y42" t="n">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="Z42" t="inlineStr">
         <is>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="AA42" t="inlineStr">
         <is>
-          <t>13/0, 15/0, 14/1, 32/0, 42/0 ,53/0  62/0,  64A/0, 64/3, 81/0</t>
+          <t>13/0, 15/0, 32/0, 42/0 ,53/0  62/0,  64A/0, 64/3, 81/0</t>
         </is>
       </c>
     </row>
@@ -4654,12 +4654,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4753,12 +4753,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4842,12 +4842,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4935,12 +4935,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -5028,12 +5028,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -5121,12 +5121,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -24999,7 +24999,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -25034,7 +25034,7 @@
       <c r="I6" t="inlineStr">
         <is>
           <t>C3:Activity-&gt;activity_raw; C4:Quantity-&gt;quantity_loa; C5:unnamed_col_5-&gt;quantity_estimated_or_total; C7:unnamed_col_7-&gt;cumulative_last_month; C9:unnamed_col_9-&gt;plan_for_month; C10:Progress for the Month-&gt;progress_for_month; C11:unnamed_col_11-&gt;today_progress; C12:Cumulative Progress-&gt;cumulative_progress; C13:Balance Progress-&gt;balance_progress; C14:Gangs working 
-May-26-&gt;gangs_working; C15:2026-05-26 00:00:00 Remarks-&gt;remarks</t>
+May-26-&gt;gangs_working; C15:2026-05-27 00:00:00 Remarks-&gt;remarks</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -25053,7 +25053,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -26607,7 +26607,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-26.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -26625,7 +26625,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="K6" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-29 10:45:17
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -1819,12 +1819,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1910,12 +1910,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2001,12 +2001,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2092,12 +2092,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2183,12 +2183,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2237,14 +2237,16 @@
         <v>34</v>
       </c>
       <c r="V18" t="n">
-        <v>13</v>
-      </c>
-      <c r="W18" t="inlineStr"/>
+        <v>14</v>
+      </c>
+      <c r="W18" t="n">
+        <v>1</v>
+      </c>
       <c r="X18" t="n">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="Y18" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="Z18" t="inlineStr"/>
       <c r="AA18" t="inlineStr"/>
@@ -2278,12 +2280,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2332,18 +2334,20 @@
         <v>34</v>
       </c>
       <c r="V19" t="n">
-        <v>13</v>
-      </c>
-      <c r="W19" t="inlineStr"/>
+        <v>14</v>
+      </c>
+      <c r="W19" t="n">
+        <v>1</v>
+      </c>
       <c r="X19" t="n">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="Y19" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="AA19" t="inlineStr"/>
@@ -2377,12 +2381,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2472,12 +2476,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2526,20 +2530,20 @@
         <v>55</v>
       </c>
       <c r="V21" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="W21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X21" t="n">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="Y21" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>14.0</t>
+          <t>13.0</t>
         </is>
       </c>
       <c r="AA21" t="inlineStr">
@@ -2577,12 +2581,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2678,12 +2682,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2743,7 +2747,7 @@
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>7.0</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="AA23" t="inlineStr"/>
@@ -2777,12 +2781,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2831,16 +2835,16 @@
         <v>20</v>
       </c>
       <c r="V24" t="n">
-        <v>6.401</v>
+        <v>8.228999999999999</v>
       </c>
       <c r="W24" t="n">
-        <v>1.327</v>
+        <v>1.828</v>
       </c>
       <c r="X24" t="n">
-        <v>18.097</v>
+        <v>19.925</v>
       </c>
       <c r="Y24" t="n">
-        <v>109.702</v>
+        <v>107.874</v>
       </c>
       <c r="Z24" t="inlineStr"/>
       <c r="AA24" t="inlineStr"/>
@@ -2874,12 +2878,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2930,9 +2934,7 @@
       <c r="V25" t="n">
         <v>7.379</v>
       </c>
-      <c r="W25" t="n">
-        <v>1.327</v>
-      </c>
+      <c r="W25" t="inlineStr"/>
       <c r="X25" t="n">
         <v>14.007</v>
       </c>
@@ -2971,12 +2973,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -5202,12 +5204,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -5303,12 +5305,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -5402,12 +5404,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -5503,12 +5505,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -5606,12 +5608,12 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -5709,12 +5711,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5783,7 +5785,7 @@
       </c>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>33/0 -34/0 - Top phase payingout under progress  + 34/0- 34/1 - PP rope passing done  + 34/1 -  34/2 - Insulator hosting done</t>
+          <t>33/0 -34/0 - Top phase payingout Done  + 34/0- 34/1 - PP rope passing done  + 34/1 -  34/2 - Insulator hosting done</t>
         </is>
       </c>
     </row>
@@ -5816,12 +5818,12 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -5915,12 +5917,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -6012,12 +6014,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -6105,12 +6107,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -8288,12 +8290,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -8385,12 +8387,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -8482,12 +8484,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -8579,12 +8581,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -8676,12 +8678,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -8773,12 +8775,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -8876,12 +8878,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -8973,12 +8975,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -9031,14 +9033,14 @@
         <v>18</v>
       </c>
       <c r="V88" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="W88" t="inlineStr"/>
       <c r="X88" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="Y88" t="n">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="Z88" t="inlineStr">
         <is>
@@ -9076,12 +9078,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -9173,12 +9175,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -9270,12 +9272,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -9367,12 +9369,12 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -9464,12 +9466,12 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -9561,12 +9563,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -9662,12 +9664,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -9763,12 +9765,12 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -9864,12 +9866,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -9965,12 +9967,12 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -10023,16 +10025,16 @@
         <v>272</v>
       </c>
       <c r="V98" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W98" t="n">
         <v>25</v>
       </c>
       <c r="X98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y98" t="n">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="Z98" t="inlineStr"/>
       <c r="AA98" t="inlineStr"/>
@@ -10066,12 +10068,12 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -10171,12 +10173,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -10264,12 +10266,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -10328,14 +10330,14 @@
         <v>30</v>
       </c>
       <c r="X101" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y101" t="n">
         <v>220</v>
       </c>
       <c r="Z101" t="inlineStr">
         <is>
-          <t>03/77</t>
+          <t>02/55</t>
         </is>
       </c>
       <c r="AA101" t="inlineStr"/>
@@ -10369,12 +10371,12 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -10468,12 +10470,12 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -10567,12 +10569,12 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -10666,12 +10668,12 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -10765,12 +10767,12 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -13537,12 +13539,12 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -13604,7 +13606,7 @@
       </c>
       <c r="Z135" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="AA135" t="inlineStr"/>
@@ -13638,12 +13640,12 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -13735,12 +13737,12 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -13836,12 +13838,12 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -13933,12 +13935,12 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -14030,12 +14032,12 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -14127,12 +14129,12 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -14214,12 +14216,12 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -14301,12 +14303,12 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -14388,12 +14390,12 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -14475,12 +14477,12 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -15607,12 +15609,12 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -15712,12 +15714,12 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -15813,12 +15815,12 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -15918,12 +15920,12 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -16019,12 +16021,12 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -16126,12 +16128,12 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -16231,12 +16233,12 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -16289,7 +16291,7 @@
       <c r="Z163" t="inlineStr"/>
       <c r="AA163" t="inlineStr">
         <is>
-          <t>33/1 to 33/0 all phase conductor paying out done.</t>
+          <t>1E/0 Jumpering completed</t>
         </is>
       </c>
     </row>
@@ -16322,12 +16324,12 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -16427,12 +16429,12 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -16528,12 +16530,12 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -16633,12 +16635,12 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -16732,12 +16734,12 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -16831,12 +16833,12 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -16940,12 +16942,12 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -17045,12 +17047,12 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -17150,12 +17152,12 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -17255,12 +17257,12 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -17340,12 +17342,12 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -17449,12 +17451,12 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -17550,12 +17552,12 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -20277,12 +20279,12 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -20376,12 +20378,12 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -20430,16 +20432,16 @@
         <v>72</v>
       </c>
       <c r="V204" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="W204" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="X204" t="n">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="Y204" t="n">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="Z204" t="inlineStr">
         <is>
@@ -20477,12 +20479,12 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -20531,16 +20533,16 @@
         <v>70</v>
       </c>
       <c r="V205" t="n">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="W205" t="n">
         <v>0</v>
       </c>
       <c r="X205" t="n">
-        <v>289</v>
+        <v>307</v>
       </c>
       <c r="Y205" t="n">
-        <v>234</v>
+        <v>216</v>
       </c>
       <c r="Z205" t="inlineStr">
         <is>
@@ -20578,12 +20580,12 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -20632,16 +20634,16 @@
         <v>75</v>
       </c>
       <c r="V206" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="W206" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X206" t="n">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="Y206" t="n">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="Z206" t="inlineStr">
         <is>
@@ -20679,12 +20681,12 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -20780,12 +20782,12 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -24782,7 +24784,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -24836,7 +24838,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -25072,7 +25074,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -25121,12 +25123,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -25428,7 +25430,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -25478,7 +25480,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O12" t="inlineStr"/>
@@ -25497,7 +25499,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -25546,7 +25548,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O13" t="inlineStr"/>
@@ -25636,7 +25638,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -25686,12 +25688,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -25781,7 +25783,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -25830,12 +25832,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -25999,7 +26001,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -26050,12 +26052,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -26428,7 +26430,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -26446,7 +26448,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
@@ -26664,7 +26666,7 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>TA 421 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 421 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -26682,12 +26684,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -26957,7 +26959,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -26975,7 +26977,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
@@ -26986,7 +26988,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>765KV TA 414 VNTL; 765KV ASOTL; Project Details; AOTL - KEC; DPR Sheet; Sheet5; Sheet3; Sheet1; Survey Anx; Soil Inv.; Survey; FDN; Erection ; Visual chart 1 ; Pile Foundation; Sheet6; Sheet4; Sheet7; Stringing Compiled; String; Crossing; Tree Enumeration; Sheet2</t>
+          <t>765KV TA 414 VNTL; 765KV ASOTL; Project Details; AOTL - KEC; DPR Sheet; Sheet5; Sheet3; Sheet1; Soil Inv.; Survey Anx; Survey; FDN; Erection ; Visual chart 1 ; Pile Foundation; Sheet6; Sheet4; Sheet7; Stringing Compiled; String; Crossing; Tree Enumeration; Sheet2</t>
         </is>
       </c>
     </row>
@@ -27014,7 +27016,7 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -27032,7 +27034,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
@@ -27189,7 +27191,7 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -27207,12 +27209,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -27360,7 +27362,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>TB 501 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 501 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -27378,12 +27380,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -27535,7 +27537,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-27.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -27553,12 +27555,12 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-29 11:48:20
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -3876,12 +3876,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3973,12 +3973,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -4070,12 +4070,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -4163,12 +4163,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -4256,12 +4256,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -4349,12 +4349,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -4405,14 +4405,14 @@
         <v>45</v>
       </c>
       <c r="V40" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="n">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="Y40" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="Z40" t="inlineStr">
         <is>
@@ -4421,7 +4421,7 @@
       </c>
       <c r="AA40" t="inlineStr">
         <is>
-          <t>38/2, 38/4, 39/0, 47/0, 52/1, 52/2, 59/0, 65/2, 66/0, 68/0, 70/0,72/0, 73/0, 75/0, 76/0, 76/1, 82/0, 87/1, 95A/0, 96/0, 96/2</t>
+          <t>38/2, 38/4, 39/0, 47/0, 52/1, 52/2, 59/0, 65/2, 66/0, 70/0,72/0, 73/0, 75/0, 76/0, 76/1, 82/0, 87/1, 96/0, 96/2</t>
         </is>
       </c>
     </row>
@@ -4454,12 +4454,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -4551,12 +4551,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4656,12 +4656,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4755,12 +4755,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4844,12 +4844,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4937,12 +4937,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -5030,12 +5030,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -5123,12 +5123,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -6200,12 +6200,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -6291,12 +6291,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -6384,12 +6384,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -6479,12 +6479,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -6572,12 +6572,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -6665,12 +6665,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -7344,12 +7344,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -7435,12 +7435,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -7526,12 +7526,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -7580,11 +7580,11 @@
         <v>40</v>
       </c>
       <c r="V73" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="W73" t="inlineStr"/>
       <c r="X73" t="n">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="Y73" t="n">
         <v>123</v>
@@ -7621,12 +7621,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -7675,11 +7675,11 @@
         <v>46</v>
       </c>
       <c r="V74" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W74" t="inlineStr"/>
       <c r="X74" t="n">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="Y74" t="n">
         <v>202</v>
@@ -7716,12 +7716,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -7811,12 +7811,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -25001,7 +25001,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -25036,7 +25036,7 @@
       <c r="I6" t="inlineStr">
         <is>
           <t>C3:Activity-&gt;activity_raw; C4:Quantity-&gt;quantity_loa; C5:unnamed_col_5-&gt;quantity_estimated_or_total; C7:unnamed_col_7-&gt;cumulative_last_month; C9:unnamed_col_9-&gt;plan_for_month; C10:Progress for the Month-&gt;progress_for_month; C11:unnamed_col_11-&gt;today_progress; C12:Cumulative Progress-&gt;cumulative_progress; C13:Balance Progress-&gt;balance_progress; C14:Gangs working 
-May-26-&gt;gangs_working; C15:2026-05-27 00:00:00 Remarks-&gt;remarks</t>
+May-26-&gt;gangs_working; C15:2026-05-28 00:00:00 Remarks-&gt;remarks</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -25055,7 +25055,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -25146,7 +25146,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -25199,7 +25199,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O8" t="inlineStr"/>
@@ -25286,7 +25286,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -25339,7 +25339,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O10" t="inlineStr"/>
@@ -26609,7 +26609,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -26627,7 +26627,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="K6" t="inlineStr"/>
@@ -26727,7 +26727,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -26745,7 +26745,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
@@ -26841,7 +26841,7 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -26859,7 +26859,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="K10" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-29 16:15:37
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -597,12 +597,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -698,12 +698,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -799,12 +799,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -900,12 +900,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1003,12 +1003,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1106,12 +1106,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1205,12 +1205,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1411,12 +1411,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1470,7 +1470,7 @@
         <v>8.6</v>
       </c>
       <c r="W10" t="n">
-        <v>2.548</v>
+        <v>0</v>
       </c>
       <c r="X10" t="n">
         <v>77.18899999999999</v>
@@ -1518,12 +1518,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1621,12 +1621,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1680,7 +1680,7 @@
         <v>8.6</v>
       </c>
       <c r="W12" t="n">
-        <v>2.548</v>
+        <v>0</v>
       </c>
       <c r="X12" t="n">
         <v>77.18899999999999</v>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -17661,12 +17661,12 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -17764,12 +17764,12 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -17867,12 +17867,12 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -17970,12 +17970,12 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -18073,12 +18073,12 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -18129,14 +18129,14 @@
         <v>30</v>
       </c>
       <c r="V181" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="W181" t="inlineStr"/>
       <c r="X181" t="n">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="Y181" t="n">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="Z181" t="inlineStr">
         <is>
@@ -18182,12 +18182,12 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -18283,12 +18283,12 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -18339,18 +18339,20 @@
         <v>30</v>
       </c>
       <c r="V183" t="n">
-        <v>19</v>
-      </c>
-      <c r="W183" t="inlineStr"/>
+        <v>20</v>
+      </c>
+      <c r="W183" t="n">
+        <v>1</v>
+      </c>
       <c r="X183" t="n">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="Y183" t="n">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="Z183" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>7.0</t>
         </is>
       </c>
       <c r="AA183" t="inlineStr">
@@ -18392,12 +18394,12 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -18499,12 +18501,12 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -18584,12 +18586,12 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -18693,12 +18695,12 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -18751,9 +18753,7 @@
       <c r="V187" t="n">
         <v>3.877</v>
       </c>
-      <c r="W187" t="n">
-        <v>0.226</v>
-      </c>
+      <c r="W187" t="inlineStr"/>
       <c r="X187" t="n">
         <v>20.923</v>
       </c>
@@ -18796,12 +18796,12 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -18889,12 +18889,12 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -18984,12 +18984,12 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -19079,12 +19079,12 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -19182,12 +19182,12 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -19285,12 +19285,12 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -19388,12 +19388,12 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -19491,12 +19491,12 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -19547,14 +19547,14 @@
         <v>11</v>
       </c>
       <c r="V195" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="W195" t="inlineStr"/>
       <c r="X195" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="Y195" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Z195" t="inlineStr">
         <is>
@@ -19600,12 +19600,12 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -19703,12 +19703,12 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -19772,7 +19772,7 @@
       </c>
       <c r="Z197" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="AA197" t="inlineStr"/>
@@ -19810,12 +19810,12 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -19905,12 +19905,12 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -19992,12 +19992,12 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -20089,12 +20089,12 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -20186,12 +20186,12 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -24705,7 +24705,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -24761,7 +24761,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -25855,7 +25855,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -25909,7 +25909,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O18" t="inlineStr"/>
@@ -25928,7 +25928,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -25982,7 +25982,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="O19" t="inlineStr"/>
@@ -26369,7 +26369,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -26387,7 +26387,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -26402,7 +26402,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>TA413_PBNTL; Visual Chart; Stringing; Stretch readiness ; Erection; L2 Plan vs Actual; Survey summary; Detailed Survey ; Check Survey ; Earthing; Tack Welding;  Final checking; Bird Guard ; Accessories; OPGW; Foundation; JUMPER Details; ROW Tracker; S-Curve FDN; S-Curve Erection; S-Curve Stringing; Supply Status; Hardware Supply; Crossing status; Tower Abstract sheet; Statutory Proposals; Tower Abstarct ; Location Summary; Foundation Daily Progress; Tower PRS abstract ; Stretch readiness  (2); Area</t>
+          <t>TA413_PBNTL; Visual Chart; Stringing; Stretch readiness ; Erection; L2 Plan vs Actual; Survey summary; Detailed Survey ; Check Survey ; Earthing; Tack Welding;  Final checking; Bird Guard ; Aviation Paint; Accessories; OPGW; Foundation; JUMPER Details; ROW Tracker; S-Curve FDN; S-Curve Erection; S-Curve Stringing; Supply Status; Hardware Supply; Crossing status; Tower Abstract sheet; Statutory Proposals; Tower Abstarct ; Location Summary; Foundation Daily Progress; Tower PRS abstract ; Stretch readiness  (2); Area</t>
         </is>
       </c>
     </row>
@@ -27423,7 +27423,7 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -27441,7 +27441,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
@@ -27480,7 +27480,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-25.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -27498,7 +27498,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto pipeline update 2026-05-31 16:18:53
</commit_message>
<xml_diff>
--- a/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
+++ b/Parquets/ProgressStatus/ProgressStatus_Output.xlsx
@@ -597,12 +597,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -698,12 +698,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -799,12 +799,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -900,12 +900,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1003,12 +1003,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1106,12 +1106,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1205,12 +1205,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1411,12 +1411,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1518,12 +1518,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1621,12 +1621,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1720,12 +1720,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1819,12 +1819,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1910,12 +1910,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2001,12 +2001,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2092,12 +2092,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2183,12 +2183,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2239,9 +2239,7 @@
       <c r="V18" t="n">
         <v>14</v>
       </c>
-      <c r="W18" t="n">
-        <v>1</v>
-      </c>
+      <c r="W18" t="inlineStr"/>
       <c r="X18" t="n">
         <v>318</v>
       </c>
@@ -2280,12 +2278,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2336,9 +2334,7 @@
       <c r="V19" t="n">
         <v>14</v>
       </c>
-      <c r="W19" t="n">
-        <v>1</v>
-      </c>
+      <c r="W19" t="inlineStr"/>
       <c r="X19" t="n">
         <v>318</v>
       </c>
@@ -2381,12 +2377,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2476,12 +2472,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2530,16 +2526,14 @@
         <v>55</v>
       </c>
       <c r="V21" t="n">
-        <v>27</v>
-      </c>
-      <c r="W21" t="n">
-        <v>2</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="W21" t="inlineStr"/>
       <c r="X21" t="n">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="Y21" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
@@ -2548,7 +2542,7 @@
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>1 gang arrived on 27.05.26</t>
+          <t>1 gang arrived on 29.05.26</t>
         </is>
       </c>
     </row>
@@ -2581,12 +2575,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2637,9 +2631,7 @@
       <c r="V22" t="n">
         <v>21</v>
       </c>
-      <c r="W22" t="n">
-        <v>2</v>
-      </c>
+      <c r="W22" t="inlineStr"/>
       <c r="X22" t="n">
         <v>100</v>
       </c>
@@ -2682,12 +2674,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2736,14 +2728,14 @@
         <v>20</v>
       </c>
       <c r="V23" t="n">
-        <v>7.379</v>
+        <v>7.622999999999999</v>
       </c>
       <c r="W23" t="inlineStr"/>
       <c r="X23" t="n">
-        <v>14.007</v>
+        <v>14.251</v>
       </c>
       <c r="Y23" t="n">
-        <v>113.792</v>
+        <v>113.548</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -2781,12 +2773,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2837,9 +2829,7 @@
       <c r="V24" t="n">
         <v>8.228999999999999</v>
       </c>
-      <c r="W24" t="n">
-        <v>1.828</v>
-      </c>
+      <c r="W24" t="inlineStr"/>
       <c r="X24" t="n">
         <v>19.925</v>
       </c>
@@ -2878,12 +2868,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2932,14 +2922,14 @@
         <v>20</v>
       </c>
       <c r="V25" t="n">
-        <v>7.379</v>
+        <v>7.622999999999999</v>
       </c>
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="n">
-        <v>14.007</v>
+        <v>14.251</v>
       </c>
       <c r="Y25" t="n">
-        <v>113.792</v>
+        <v>113.548</v>
       </c>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="inlineStr"/>
@@ -2973,12 +2963,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -3066,12 +3056,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -3167,12 +3157,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -3268,12 +3258,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3369,12 +3359,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -3426,7 +3416,7 @@
         <v>4.41</v>
       </c>
       <c r="W30" t="n">
-        <v>0.359</v>
+        <v>0</v>
       </c>
       <c r="X30" t="n">
         <v>111.133</v>
@@ -3470,12 +3460,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 418 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3537,7 +3527,7 @@
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AA31" t="inlineStr"/>
@@ -3571,12 +3561,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 418 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3638,7 +3628,7 @@
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AA32" t="inlineStr"/>
@@ -3672,12 +3662,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 418 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3739,7 +3729,7 @@
       </c>
       <c r="Z33" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AA33" t="inlineStr"/>
@@ -3773,12 +3763,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 418 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3827,23 +3817,23 @@
         <v>11.89</v>
       </c>
       <c r="V34" t="n">
-        <v>3.963</v>
+        <v>5.84</v>
       </c>
       <c r="W34" t="inlineStr"/>
       <c r="X34" t="n">
-        <v>27.705</v>
+        <v>29.582</v>
       </c>
       <c r="Y34" t="n">
-        <v>20.135</v>
+        <v>18.258</v>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>*Work Front Required for HotLine Gang</t>
+          <t>*Work Front Required for Hotline Gang</t>
         </is>
       </c>
     </row>
@@ -3876,12 +3866,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3973,12 +3963,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -4070,12 +4060,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -4163,12 +4153,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -4256,12 +4246,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -4349,12 +4339,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -4454,12 +4444,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -4551,12 +4541,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4623,7 +4613,7 @@
       </c>
       <c r="AA42" t="inlineStr">
         <is>
-          <t>13/0, 15/0, 32/0, 42/0 ,53/0  62/0,  64A/0, 64/3, 81/0</t>
+          <t>13/0, 15/0, 32/0, 42/0 ,53/0, 62/0,  64A/0, 64/3, 81/0</t>
         </is>
       </c>
     </row>
@@ -4656,12 +4646,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -4755,12 +4745,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4844,12 +4834,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4937,12 +4927,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -5030,12 +5020,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -5123,12 +5113,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -6200,12 +6190,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-29.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -6291,12 +6281,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-29.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -6384,12 +6374,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-29.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -6438,11 +6428,11 @@
         <v>29</v>
       </c>
       <c r="V61" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W61" t="inlineStr"/>
       <c r="X61" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="Y61" t="n">
         <v>47</v>
@@ -6479,12 +6469,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-29.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -6572,12 +6562,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-29.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -6665,12 +6655,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-29.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -7344,12 +7334,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-29.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -7435,12 +7425,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-29.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -7526,12 +7516,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-29.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -7580,11 +7570,11 @@
         <v>40</v>
       </c>
       <c r="V73" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="W73" t="inlineStr"/>
       <c r="X73" t="n">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="Y73" t="n">
         <v>123</v>
@@ -7621,12 +7611,12 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-29.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -7675,11 +7665,11 @@
         <v>46</v>
       </c>
       <c r="V74" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W74" t="inlineStr"/>
       <c r="X74" t="n">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="Y74" t="n">
         <v>202</v>
@@ -7716,12 +7706,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-29.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -7770,11 +7760,11 @@
         <v>38</v>
       </c>
       <c r="V75" t="n">
-        <v>10.629</v>
+        <v>12.064</v>
       </c>
       <c r="W75" t="inlineStr"/>
       <c r="X75" t="n">
-        <v>54.197</v>
+        <v>55.632</v>
       </c>
       <c r="Y75" t="n">
         <v>179.432</v>
@@ -7811,12 +7801,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-29.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -8290,12 +8280,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -8387,12 +8377,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -8484,12 +8474,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -8581,12 +8571,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -8678,12 +8668,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -8775,12 +8765,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -8878,12 +8868,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -8975,12 +8965,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -9078,12 +9068,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -9175,12 +9165,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -9272,12 +9262,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -9369,12 +9359,12 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -9466,12 +9456,12 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -9563,12 +9553,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -9664,12 +9654,12 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -9765,12 +9755,12 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -9866,12 +9856,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -9967,12 +9957,12 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -10031,7 +10021,7 @@
         <v>25</v>
       </c>
       <c r="X98" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y98" t="n">
         <v>309</v>
@@ -10068,12 +10058,12 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -10126,7 +10116,7 @@
         <v>272</v>
       </c>
       <c r="V99" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W99" t="n">
         <v>25</v>
@@ -10135,7 +10125,7 @@
         <v>0</v>
       </c>
       <c r="Y99" t="n">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="Z99" t="inlineStr">
         <is>
@@ -10173,12 +10163,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -10266,12 +10256,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -10324,16 +10314,16 @@
         <v>210</v>
       </c>
       <c r="V101" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W101" t="n">
         <v>30</v>
       </c>
       <c r="X101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y101" t="n">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="Z101" t="inlineStr">
         <is>
@@ -10371,12 +10361,12 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -10470,12 +10460,12 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -10569,12 +10559,12 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -10668,12 +10658,12 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -10767,12 +10757,12 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -13539,12 +13529,12 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -13593,16 +13583,16 @@
         <v>40</v>
       </c>
       <c r="V135" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="W135" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X135" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="Y135" t="n">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="Z135" t="inlineStr">
         <is>
@@ -13640,12 +13630,12 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -13694,16 +13684,16 @@
         <v>40</v>
       </c>
       <c r="V136" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="W136" t="n">
         <v>0</v>
       </c>
       <c r="X136" t="n">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="Y136" t="n">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="Z136" t="inlineStr"/>
       <c r="AA136" t="inlineStr"/>
@@ -13737,12 +13727,12 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -13838,12 +13828,12 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -13935,12 +13925,12 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -14032,12 +14022,12 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -14129,12 +14119,12 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -14216,12 +14206,12 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -14303,12 +14293,12 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -14390,12 +14380,12 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -14477,12 +14467,12 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -14558,12 +14548,12 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -14657,12 +14647,12 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -14754,12 +14744,12 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -14839,12 +14829,12 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -14924,12 +14914,12 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -14984,16 +14974,16 @@
         <v>35</v>
       </c>
       <c r="V150" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="W150" t="n">
         <v>1</v>
       </c>
       <c r="X150" t="n">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="Y150" t="n">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="Z150" t="inlineStr">
         <is>
@@ -15031,12 +15021,12 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -15132,12 +15122,12 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -15221,12 +15211,12 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -15310,12 +15300,12 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -15405,12 +15395,12 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -15502,12 +15492,12 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -15562,16 +15552,14 @@
         <v>40</v>
       </c>
       <c r="V156" t="n">
-        <v>25</v>
-      </c>
-      <c r="W156" t="n">
-        <v>1</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="W156" t="inlineStr"/>
       <c r="X156" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="Y156" t="n">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="Z156" t="inlineStr">
         <is>
@@ -17661,12 +17649,12 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -17764,12 +17752,12 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -17867,12 +17855,12 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -17970,12 +17958,12 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -18073,12 +18061,12 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -18129,18 +18117,20 @@
         <v>30</v>
       </c>
       <c r="V181" t="n">
-        <v>17</v>
-      </c>
-      <c r="W181" t="inlineStr"/>
+        <v>18</v>
+      </c>
+      <c r="W181" t="n">
+        <v>1</v>
+      </c>
       <c r="X181" t="n">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Y181" t="n">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="Z181" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="AA181" t="inlineStr">
@@ -18182,12 +18172,12 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -18283,12 +18273,12 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -18342,7 +18332,7 @@
         <v>20</v>
       </c>
       <c r="W183" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X183" t="n">
         <v>214</v>
@@ -18394,12 +18384,12 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -18501,12 +18491,12 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -18586,12 +18576,12 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -18642,14 +18632,14 @@
         <v>15.147</v>
       </c>
       <c r="V186" t="n">
-        <v>3.877</v>
+        <v>4.314</v>
       </c>
       <c r="W186" t="inlineStr"/>
       <c r="X186" t="n">
-        <v>21.36</v>
+        <v>21.797</v>
       </c>
       <c r="Y186" t="n">
-        <v>167.318</v>
+        <v>166.881</v>
       </c>
       <c r="Z186" t="inlineStr">
         <is>
@@ -18695,12 +18685,12 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -18751,14 +18741,16 @@
         <v>15.147</v>
       </c>
       <c r="V187" t="n">
-        <v>3.877</v>
-      </c>
-      <c r="W187" t="inlineStr"/>
+        <v>4.314</v>
+      </c>
+      <c r="W187" t="n">
+        <v>0.437</v>
+      </c>
       <c r="X187" t="n">
-        <v>20.923</v>
+        <v>21.36</v>
       </c>
       <c r="Y187" t="n">
-        <v>167.755</v>
+        <v>167.318</v>
       </c>
       <c r="Z187" t="inlineStr"/>
       <c r="AA187" t="inlineStr"/>
@@ -18796,12 +18788,12 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -18889,12 +18881,12 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -18984,12 +18976,12 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -19079,12 +19071,12 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -19182,12 +19174,12 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -19285,12 +19277,12 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -19388,12 +19380,12 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -19491,12 +19483,12 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -19558,12 +19550,12 @@
       </c>
       <c r="Z195" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="AA195" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>20.0</t>
         </is>
       </c>
     </row>
@@ -19600,12 +19592,12 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -19703,12 +19695,12 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -19770,11 +19762,7 @@
       <c r="Y197" t="n">
         <v>40</v>
       </c>
-      <c r="Z197" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
+      <c r="Z197" t="inlineStr"/>
       <c r="AA197" t="inlineStr"/>
     </row>
     <row r="198">
@@ -19810,12 +19798,12 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -19905,12 +19893,12 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -19992,12 +19980,12 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -20089,12 +20077,12 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -20186,12 +20174,12 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -20279,12 +20267,12 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -20378,12 +20366,12 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -20432,20 +20420,20 @@
         <v>72</v>
       </c>
       <c r="V204" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="W204" t="n">
         <v>4</v>
       </c>
       <c r="X204" t="n">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="Y204" t="n">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="Z204" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>29</t>
         </is>
       </c>
       <c r="AA204" t="inlineStr"/>
@@ -20479,12 +20467,12 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -20533,16 +20521,16 @@
         <v>70</v>
       </c>
       <c r="V205" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="W205" t="n">
         <v>0</v>
       </c>
       <c r="X205" t="n">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="Y205" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="Z205" t="inlineStr">
         <is>
@@ -20580,12 +20568,12 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -20634,16 +20622,16 @@
         <v>75</v>
       </c>
       <c r="V206" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="W206" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X206" t="n">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="Y206" t="n">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="Z206" t="inlineStr">
         <is>
@@ -20681,12 +20669,12 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -20782,12 +20770,12 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -24705,7 +24693,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -24761,7 +24749,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -24784,7 +24772,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -24838,7 +24826,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O3" t="inlineStr"/>
@@ -24857,7 +24845,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -24906,17 +24894,17 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>MATCH</t>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -24929,7 +24917,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 418 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -24978,17 +24966,17 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -25001,7 +24989,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -25036,7 +25024,7 @@
       <c r="I6" t="inlineStr">
         <is>
           <t>C3:Activity-&gt;activity_raw; C4:Quantity-&gt;quantity_loa; C5:unnamed_col_5-&gt;quantity_estimated_or_total; C7:unnamed_col_7-&gt;cumulative_last_month; C9:unnamed_col_9-&gt;plan_for_month; C10:Progress for the Month-&gt;progress_for_month; C11:unnamed_col_11-&gt;today_progress; C12:Cumulative Progress-&gt;cumulative_progress; C13:Balance Progress-&gt;balance_progress; C14:Gangs working 
-May-26-&gt;gangs_working; C15:2026-05-28 00:00:00 Remarks-&gt;remarks</t>
+May-26-&gt;gangs_working; C15:2026-05-29 00:00:00 Remarks-&gt;remarks</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -25055,7 +25043,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -25146,7 +25134,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-29.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -25199,7 +25187,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O8" t="inlineStr"/>
@@ -25286,7 +25274,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-29.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -25339,7 +25327,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O10" t="inlineStr"/>
@@ -25430,7 +25418,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -25480,7 +25468,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O12" t="inlineStr"/>
@@ -25499,7 +25487,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -25548,7 +25536,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O13" t="inlineStr"/>
@@ -25638,7 +25626,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -25688,12 +25676,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -25711,7 +25699,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -25760,17 +25748,17 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -25855,7 +25843,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -25909,7 +25897,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O18" t="inlineStr"/>
@@ -25928,7 +25916,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -25982,7 +25970,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O19" t="inlineStr"/>
@@ -26001,7 +25989,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -26052,12 +26040,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -26369,7 +26357,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>TA 413 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 413 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -26387,7 +26375,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -26430,7 +26418,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TA 414 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 414 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -26448,7 +26436,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
@@ -26459,7 +26447,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Project Details; 765KV TA 414 VNTL; VNTL - KEC; DPR Sheet; Sheet5; Sheet3; Sheet1; FDN; FDN Completed; Erection ; Erection Completed ; Erection Compiled; Stringing; Stringing Completed; Stringing Compiled; Sheet6; Sheet4; Sheet7; Visual chart; Pile Fdn; Crossing; Sheet2; Survey; Soil Inv.; Survey Anx</t>
+          <t>Project Details; 765KV TA 414 VNTL; VNTL - KEC; DPR Sheet; Sheet5; Sheet3; Sheet1; FDN; FDN Completed; Erection ; Erection Completed ; Erection Compiled; Stringing; Stringing Completed; Sheet6; Sheet4; Sheet7; Stringing Compiled; Visual chart; Pile Fdn; Crossing; Sheet2; Survey; Soil Inv.; Survey Anx</t>
         </is>
       </c>
     </row>
@@ -26487,7 +26475,7 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>TA 416 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 416 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -26505,17 +26493,17 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>MATCH</t>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -26548,7 +26536,7 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>TA 418 - DPR - 2026-05-21.xlsx</t>
+          <t>TA 418 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -26566,22 +26554,22 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>MASTER SHEET; Progress; Erection Compiled; Stringing Compiled; Visual Chart; ROW TRACKER; PENDING FDN DETAILS; TSE-MANUAL-LT-11KV-33KV Details; Crossing Details; Project Details; TS; TS (2)</t>
+          <t>MASTER SHEET; Progress; Erection Completed; Stringing Completed; Visual Chart; ROW TRACKER; PENDING FDN DETAILS; TSE-MANUAL-LT-11KV-33KV Details; Crossing Details; Project Details; TS; TS (2)</t>
         </is>
       </c>
     </row>
@@ -26609,7 +26597,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TA 419 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 419 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -26627,7 +26615,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="K6" t="inlineStr"/>
@@ -26727,7 +26715,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TA 504 - DPR - 2026-05-29.xlsx</t>
+          <t>TA 504 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -26745,7 +26733,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
@@ -26841,7 +26829,7 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>TA 506 - DPR - 2026-05-29.xlsx</t>
+          <t>TA 506 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -26859,7 +26847,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="K10" t="inlineStr"/>
@@ -26959,7 +26947,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>TA 510 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 510 - DPR - 2026-05-29.xlsx</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -26977,7 +26965,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
@@ -27016,7 +27004,7 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>TA 512 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 512 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -27034,7 +27022,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
@@ -27191,7 +27179,7 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>TA 601 - DPR - 2026-05-28.xlsx</t>
+          <t>TA 601 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -27209,12 +27197,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -27252,7 +27240,7 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>TA 602 - DPR - 2026-05-27.xlsx</t>
+          <t>TA 602 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -27270,17 +27258,17 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -27423,7 +27411,7 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>TB 507 [MAIN] - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 [MAIN] - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -27441,7 +27429,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
@@ -27480,7 +27468,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>TB 507 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 507 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -27498,7 +27486,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>
@@ -27537,7 +27525,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>TB 605 - DPR - 2026-05-28.xlsx</t>
+          <t>TB 605 - DPR - 2026-05-30.xlsx</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -27555,12 +27543,12 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">

</xml_diff>